<commit_message>
new Contact, Careers, Home, backToTop, vacancy
</commit_message>
<xml_diff>
--- a/public/procurement.xlsx
+++ b/public/procurement.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lka\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6EF2FC24-8428-43AE-920B-1F71F78F97F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19AD3BCB-6882-40CB-BE56-C90C1CB4DE3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="633" uniqueCount="248">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="597" uniqueCount="234">
   <si>
     <t>№ п/п</t>
   </si>
@@ -54,21 +54,21 @@
     <t>ЛГУП-7511</t>
   </si>
   <si>
+    <t>ЛГУП-7564</t>
+  </si>
+  <si>
+    <t>м</t>
+  </si>
+  <si>
     <t>кг</t>
   </si>
   <si>
-    <t>ЛГУП-7564</t>
-  </si>
-  <si>
     <t>м2</t>
   </si>
   <si>
     <t>Лист S=6 Ст.09Г2С ГОСТ 19281-89</t>
   </si>
   <si>
-    <t>м</t>
-  </si>
-  <si>
     <t>Ящик пластиковый396х297х280</t>
   </si>
   <si>
@@ -96,15 +96,21 @@
     <t>Ремонт двери 1900х1000мм(уст.ка вент. решеток, установка цепи и фиксатора, покраска)</t>
   </si>
   <si>
+    <t>Лампа индикации ADDS D22 LED белая 220В AC/DC ЛK-22 IP55 25152DEK Dekraft</t>
+  </si>
+  <si>
+    <t>ЛГУП-7654</t>
+  </si>
+  <si>
     <t>Резьбовой крепежный элемент с наружной резьбой РКН-20 У2 IP54 ЗЭТА</t>
   </si>
   <si>
-    <t>ЛГУП-7654</t>
-  </si>
-  <si>
     <t>Электроприв четвер.взры. ГЗ-ОФВ-300/28М 1х220 DN80PN63 L=452 УХЛ (исп. фл. J)</t>
   </si>
   <si>
+    <t>Аварийное освещение Вега 60 с БАП 2Ex Тех 1ExmbIIC T6 Gb X, IP65</t>
+  </si>
+  <si>
     <t>Пломба 1-6х10-АД-1М ГОСТ 18677-73</t>
   </si>
   <si>
@@ -120,24 +126,21 @@
     <t>мм</t>
   </si>
   <si>
+    <t>Извещатель пожарный тепловой взрывозащищенный 101-07е 1Ex db [ia Ga] IIC Т4 Gb Х IP66</t>
+  </si>
+  <si>
     <t>Винт для обеспечения электрического контакта крышек ( М 5 х 8) арт.CM030508</t>
   </si>
   <si>
-    <t>Аварийное освещение Вега 60 с БАП 2Ex Тех 1ExmbIIC T6 Gb X, IP65</t>
-  </si>
-  <si>
-    <t>Извещатель пожарный тепловой взрывозащищенный 101-07е 1Ex db [ia Ga] IIC Т4 Gb Х IP66</t>
-  </si>
-  <si>
-    <t>Лампа индикации ADDS D22 LED белая 220В AC/DC ЛK-22 IP55 25152DEK Dekraft</t>
+    <t>Рулетка  7,5м х 25мм обрезиненный корпус (3 фиксатора, зацеп с магнитом)</t>
+  </si>
+  <si>
+    <t>ЛГУП-7867</t>
   </si>
   <si>
     <t>Бита (вставка) Spline М 8  L=30мм</t>
   </si>
   <si>
-    <t>ЛГУП-7867</t>
-  </si>
-  <si>
     <t>Ветошь /рул./</t>
   </si>
   <si>
@@ -165,27 +168,27 @@
     <t>Перчатки 4нит. 10кл. (черные) (пара)</t>
   </si>
   <si>
-    <t>Рулетка  7,5м х 25мм обрезиненный корпус (3 фиксатора, зацеп с магнитом)</t>
+    <t>Маркер по металлу черный тонкий</t>
+  </si>
+  <si>
+    <t>НТУП-018192</t>
+  </si>
+  <si>
+    <t>Маркер по металлу белый</t>
   </si>
   <si>
     <t>Маркер по металлу красный</t>
   </si>
   <si>
-    <t>НТУП-018192</t>
-  </si>
-  <si>
-    <t>Маркер по металлу белый</t>
-  </si>
-  <si>
-    <t>Маркер по металлу черный тонкий</t>
+    <t>Паронит 3 мм</t>
+  </si>
+  <si>
+    <t>лист</t>
   </si>
   <si>
     <t>Паронит 2мм</t>
   </si>
   <si>
-    <t>лист</t>
-  </si>
-  <si>
     <t>Ключи обмедненные</t>
   </si>
   <si>
@@ -195,9 +198,6 @@
     <t>Мел сварщика белый</t>
   </si>
   <si>
-    <t>Паронит 3 мм</t>
-  </si>
-  <si>
     <t>ЛГУП-7998</t>
   </si>
   <si>
@@ -216,84 +216,21 @@
     <t>ЛГУП-8015</t>
   </si>
   <si>
-    <t>Пластина R390-11 11т308 М -РМ 1130</t>
-  </si>
-  <si>
-    <t>ЛГУП-8023</t>
-  </si>
-  <si>
-    <t>НТУП-018253</t>
-  </si>
-  <si>
-    <t>Отвод 57х6, 09Г2С ГОСТ 17375-2001</t>
-  </si>
-  <si>
-    <t>отвод 89х8, 09Г2С ГОСТ 17375-2001</t>
-  </si>
-  <si>
-    <t>Отвод 114х8 ст 09Г2с</t>
-  </si>
-  <si>
-    <t>Отвод 159х8, 09Г2С ГОСТ 17375-2001</t>
-  </si>
-  <si>
-    <t>Заглушка 114х8 09Г2С ГОСТ 17379-2001</t>
-  </si>
-  <si>
-    <t>Отвод 219х8</t>
-  </si>
-  <si>
-    <t>Заглушка 57х6 ст.09Г2С ГОСТ 17379-01</t>
-  </si>
-  <si>
-    <t>Отвод 76х8, ст09г2с ГОСТ 17375-2001</t>
-  </si>
-  <si>
-    <t>НТУП-018254</t>
-  </si>
-  <si>
-    <t>Швеллер 16П (12м) ГОСТ  8240-97</t>
-  </si>
-  <si>
-    <t>Труба 159x8,0 ГОСТ 8732-78/09Г2С ГОСТ 8731-74</t>
-  </si>
-  <si>
-    <t>Труба 114x8,0 ГОСТ 8732-78/09Г2С ГОСТ 8731-74</t>
+    <t>Шестиграник 27-h12 ГОСТ 8560-78/(ст.13ХФА)</t>
+  </si>
+  <si>
+    <t>ЛГ00-000047</t>
+  </si>
+  <si>
+    <t>ЛГ00-000048</t>
+  </si>
+  <si>
+    <t>Смеси асфальтобетонные плотные мелкозернистые, тип А, марка 1</t>
   </si>
   <si>
     <t>т</t>
   </si>
   <si>
-    <t>Труба 76х8 ст. 09Г2С ГОСТ 8732-78</t>
-  </si>
-  <si>
-    <t>т</t>
-  </si>
-  <si>
-    <t>Шестиграник 27-h12 ГОСТ 8560-78/(ст.13ХФА)</t>
-  </si>
-  <si>
-    <t>ЛГ00-000047</t>
-  </si>
-  <si>
-    <t>Ноутбук</t>
-  </si>
-  <si>
-    <t>НТУП-018276</t>
-  </si>
-  <si>
-    <t>Мышь проводная</t>
-  </si>
-  <si>
-    <t>ЛГУП-8039</t>
-  </si>
-  <si>
-    <t>ЛГ00-000048</t>
-  </si>
-  <si>
-    <t>Смеси асфальтобетонные плотные мелкозернистые, тип А, марка 1</t>
-  </si>
-  <si>
     <t>ЛГУП-8043</t>
   </si>
   <si>
@@ -303,126 +240,156 @@
     <t>ЛГУП-8046</t>
   </si>
   <si>
-    <t>Отвод 90-32х4 ст.12Х18Н10Т ГОСТ 17375-2001</t>
-  </si>
-  <si>
-    <t>ЛГУП-8049</t>
-  </si>
-  <si>
-    <t>Труба D32х4 ГОСТ 8732-78/ 12Х18Н10Т ГОСТ 5632-2014</t>
+    <t>Индустриальное масло  Gazpromneft  Industrial 40 ( И-40А ) 205л</t>
+  </si>
+  <si>
+    <t>ЛГУП-8058</t>
+  </si>
+  <si>
+    <t>Кран шаровый ДУ80 Ру 40 под приварку</t>
+  </si>
+  <si>
+    <t>НТУП-018299</t>
+  </si>
+  <si>
+    <t>ЛГУП-8060</t>
+  </si>
+  <si>
+    <t>ЛГУП-8061</t>
+  </si>
+  <si>
+    <t>(не исп1) шт</t>
+  </si>
+  <si>
+    <t>Шайба 5Л ГОСТ 6402-70</t>
+  </si>
+  <si>
+    <t>ЛГУП-8062</t>
+  </si>
+  <si>
+    <t>Коробка соединительно-разветвительная взрывозащищенная КСРВ-2-2/0-К</t>
+  </si>
+  <si>
+    <t>Текстолит 4мм (90х60)</t>
+  </si>
+  <si>
+    <t>Саморез-шуруп острый (оцинк.) 2,2х4,5 ГОСТ 1144-80</t>
+  </si>
+  <si>
+    <t>Стойка для печатных плат (шестигр., латунь) М4, 27мм ГОСТ 20862-81</t>
+  </si>
+  <si>
+    <t>Гофрокороб 395*155*155</t>
+  </si>
+  <si>
+    <t>Проволока КО 1,0 ГОСТ 792-67</t>
+  </si>
+  <si>
+    <t>Лента упаковочная полипропиленовая 12х0,6мм</t>
+  </si>
+  <si>
+    <t>Круг D30 Ст.20 ГОСТ 1050-88</t>
+  </si>
+  <si>
+    <t>Круг D24 Ст.45 ГОСТ 1050-88</t>
+  </si>
+  <si>
+    <t>Круг D20 Ст.35 ГОСТ 1050-88</t>
+  </si>
+  <si>
+    <t>Круг D32 Ст. 45 ГОСТ 1050-88</t>
+  </si>
+  <si>
+    <t>Сетка полутомпаковая 008Н Л80 ГОСТ 6613-86</t>
+  </si>
+  <si>
+    <t>Проволока D1.8 Ст.60C2А ГОСТ14963-78</t>
+  </si>
+  <si>
+    <t>Лист Б-ПН-5 ГОСТ 19903/20-ТВ1-М1-КИ-ТО ГОСТ1577</t>
+  </si>
+  <si>
+    <t>Лист Б-ПН-5 ГОСТ 19903-74 / 2-IV-Н Ст.3кп ГОСТ 16523-97 (кг)</t>
   </si>
   <si>
     <t>Лист Б-ПН-10 ГОСТ 19903-74 / 2-IV-Н Ст.3кп ГОСТ 16523-97 (кг)</t>
   </si>
   <si>
-    <t>Лист Б-ПН-5 ГОСТ 19903-74 / 2-IV-Н Ст.3кп ГОСТ 16523-97 (кг)</t>
-  </si>
-  <si>
-    <t>Лист Б-ПН-5 ГОСТ 19903/20-ТВ1-М1-КИ-ТО ГОСТ1577</t>
-  </si>
-  <si>
-    <t>Сетка полутомпаковая 008Н Л80 ГОСТ 6613-86</t>
-  </si>
-  <si>
-    <t>Проволока D1.8 Ст.60C2А ГОСТ14963-78</t>
-  </si>
-  <si>
-    <t>Круг D20 Ст.35 ГОСТ 1050-88</t>
+    <t>Лист алюм. анод. сатин (черн/бел) 1,0</t>
   </si>
   <si>
     <t>Круг D90 Ст.35 ГОСт1050-88</t>
   </si>
   <si>
-    <t>Круг D24 Ст.45 ГОСТ 1050-88</t>
-  </si>
-  <si>
-    <t>Круг D30 Ст.20 ГОСТ 1050-88</t>
-  </si>
-  <si>
-    <t>Круг D32 Ст. 45 ГОСТ 1050-88</t>
+    <t>Круг D90 Ст.20Х13 ГОСТ 5632-72</t>
+  </si>
+  <si>
+    <t>Круг D80 Ст.45 ГОСТ 1050-88</t>
+  </si>
+  <si>
+    <t>Круг D18 Ст.20Х13 ГОСТ 5949-75</t>
+  </si>
+  <si>
+    <t>Круг D110 Ст.12Х18Н10Т ГОСТ 5949-75</t>
+  </si>
+  <si>
+    <t>Круг D100 Ст.35 ГOСТ 1050-2013</t>
+  </si>
+  <si>
+    <t>Круг D75 Ст.20 ГОСТ 1050-88</t>
+  </si>
+  <si>
+    <t>Круг D70 Ст.20Х13 ГОСТ5632-72</t>
+  </si>
+  <si>
+    <t>Круг D65 Ст.35 ГОСТ 1050-88</t>
+  </si>
+  <si>
+    <t>Круг D65 Ст.3 ГОСТ 535-2005</t>
+  </si>
+  <si>
+    <t>Круг D60 Ст.35 ГОСТ 1050-88</t>
   </si>
   <si>
     <t>Круг D4 Ст.10 ГОСТ 1050-88</t>
   </si>
   <si>
-    <t>Гофрокороб 395*155*155</t>
+    <t>Круг D45 Ст.45 ГОСТ 1050-2013</t>
+  </si>
+  <si>
+    <t>Круг D45 Ст.3 ГОСТ 535-2005</t>
+  </si>
+  <si>
+    <t>Круг D80 Ст.35 ГОСТ 1050-88</t>
+  </si>
+  <si>
+    <t>Круг D75 Ст.35 ГОСТ 1050-88</t>
+  </si>
+  <si>
+    <t>Круг D75 Ст.20Х13 ГОСТ 5632-72</t>
   </si>
   <si>
     <t>Круг D42 Ст.14Х17Н2 ГОСТ 5949-75</t>
   </si>
   <si>
-    <t>Круг D80 Ст.45 ГОСТ 1050-88</t>
-  </si>
-  <si>
-    <t>Круг D90 Ст.20Х13 ГОСТ 5632-72</t>
-  </si>
-  <si>
-    <t>Круг D18 Ст.20Х13 ГОСТ 5949-75</t>
-  </si>
-  <si>
-    <t>Круг D110 Ст.12Х18Н10Т ГОСТ 5949-75</t>
-  </si>
-  <si>
-    <t>Круг D100 Ст.35 ГOСТ 1050-2013</t>
-  </si>
-  <si>
-    <t>Круг D75 Ст.20 ГОСТ 1050-88</t>
-  </si>
-  <si>
-    <t>Лист алюм. анод. сатин (черн/бел) 1,0</t>
-  </si>
-  <si>
     <t>Круг D20 Ст.20 ГОСТ 1050-88</t>
   </si>
   <si>
-    <t>Круг D75 Ст.20Х13 ГОСТ 5632-72</t>
-  </si>
-  <si>
-    <t>Круг D75 Ст.35 ГОСТ 1050-88</t>
-  </si>
-  <si>
-    <t>Проволока КО 1,0 ГОСТ 792-67</t>
-  </si>
-  <si>
-    <t>Лента упаковочная полипропиленовая 12х0,6мм</t>
-  </si>
-  <si>
-    <t>Круг D80 Ст.35 ГОСТ 1050-88</t>
-  </si>
-  <si>
-    <t>Круг D45 Ст.3 ГОСТ 535-2005</t>
-  </si>
-  <si>
-    <t>Круг D45 Ст.45 ГОСТ 1050-2013</t>
-  </si>
-  <si>
-    <t>Круг D60 Ст.35 ГОСТ 1050-88</t>
-  </si>
-  <si>
-    <t>Круг D65 Ст.3 ГОСТ 535-2005</t>
-  </si>
-  <si>
-    <t>Круг D65 Ст.35 ГОСТ 1050-88</t>
-  </si>
-  <si>
-    <t>Круг D70 Ст.20Х13 ГОСТ5632-72</t>
+    <t>Днище 377х12-09Г2С ГОСТ 6533-78</t>
+  </si>
+  <si>
+    <t>Днище 219х4-25 16ГС-3 ГОСТ 6533-78</t>
+  </si>
+  <si>
+    <t>Днище 1020х14-09Г2С ГОСТ 6533-78</t>
+  </si>
+  <si>
+    <t>Днище 820х12-09Г2С ГОСТ 6533-78</t>
   </si>
   <si>
     <t>Днище 530х12-09Г2С ГОСТ 6533-78</t>
   </si>
   <si>
-    <t>Днище 820х12-09Г2С ГОСТ 6533-78</t>
-  </si>
-  <si>
-    <t>Днище 377х12-09Г2С ГОСТ 6533-78</t>
-  </si>
-  <si>
-    <t>Днище 219х4-25 16ГС-3 ГОСТ 6533-78</t>
-  </si>
-  <si>
-    <t>Днище 1020х14-09Г2С ГОСТ 6533-78</t>
-  </si>
-  <si>
     <t>Днище 720х12-09Г2С ГОСТ 6533-78</t>
   </si>
   <si>
@@ -459,6 +426,72 @@
     <t>Пластина анкерная 120</t>
   </si>
   <si>
+    <t>Пластина для заземления PTCE арт. 37501</t>
+  </si>
+  <si>
+    <t>Плата печатная ПСМ.11.00.01.01-02</t>
+  </si>
+  <si>
+    <t>Плата питания ПСМ.11.00.00.01-02</t>
+  </si>
+  <si>
+    <t>Угол горизонтальный CPO 90 (50 х 50)</t>
+  </si>
+  <si>
+    <t>Уплотнительный модуль МКС 20/О 5-14мм</t>
+  </si>
+  <si>
+    <t>Уплотнительный модуль МКС 40/Ø 17-34 мм</t>
+  </si>
+  <si>
+    <t>Наконечник НВИ 2-5 вилка 1,5-2,5мм SQ0503-0005 TDM</t>
+  </si>
+  <si>
+    <t>Припой с канифолью ПОС 61 d=1,0мм ГОСТ 21931-76 (Sn61; Pb39)</t>
+  </si>
+  <si>
+    <t>Держатель проводника Rd8, DEHNGRIP NIRO h20 с отв.8мм М6</t>
+  </si>
+  <si>
+    <t>Диод КД209А ТТЗ.362.008 ТУ</t>
+  </si>
+  <si>
+    <t>Заглушка  25х25 для трубы профильной ПВД черная</t>
+  </si>
+  <si>
+    <t>Заглушка 10707 Legrand DPL 65х195</t>
+  </si>
+  <si>
+    <t>Лента самоклеящаяся уплотнительная ППЭ 5х15 МКС</t>
+  </si>
+  <si>
+    <t>Трубка для фильтра 1/4" Гейзер</t>
+  </si>
+  <si>
+    <t>MV-клемма проводника Rd8</t>
+  </si>
+  <si>
+    <t>Кабель-канал 10453 Legrand DPL 195х65 (2м)</t>
+  </si>
+  <si>
+    <t>Компрессионный блок МКС КБ 120</t>
+  </si>
+  <si>
+    <t>Консоль с опорой ML 300мм (шт)</t>
+  </si>
+  <si>
+    <t>Коробка клеммная МТ Р307(-60+40) 2-6х20НК(А)-1х20НК(В)-6х20НК(С)-4х26(П) 1ЕхеLLCGbXT6, ip66</t>
+  </si>
+  <si>
+    <t>Коробка клеммная МТ Р402(-60+40)12-2х20НК(А)-2х20НК(С)-1,5х11(П), 1ЕхеLLCGbXT6, ip66, 110х75х55</t>
+  </si>
+  <si>
+    <t>Коробка клеммная МТ Р403(-60+40) 2-4х20НК(А)-4х20НК(С)-2,5х20(П),1ЕхеLLCGbXT6, ip66, 160х175х55</t>
+  </si>
+  <si>
+    <t>Коробка клеммная МТ Р407(-60+40) 2-8х20НК(А)-8х20НК(С)-2,5х31(П),1ЕхеLLCGbXT6, ip66, 220х120х90</t>
+  </si>
+  <si>
     <t>Короб ПВХ 40х40 мм</t>
   </si>
   <si>
@@ -513,61 +546,34 @@
     <t>Металлорукав в ПВХ изоляции РЗ-ЦП-15</t>
   </si>
   <si>
-    <t>Наконечник НВИ 2-5 вилка 1,5-2,5мм SQ0503-0005 TDM</t>
-  </si>
-  <si>
-    <t>MV-клемма проводника Rd8</t>
-  </si>
-  <si>
-    <t>Припой с канифолью ПОС 61 d=1,0мм ГОСТ 21931-76 (Sn61; Pb39)</t>
-  </si>
-  <si>
-    <t>Лента самоклеящаяся уплотнительная ППЭ 5х15 МКС</t>
-  </si>
-  <si>
-    <t>Трубка для фильтра 1/4" Гейзер</t>
-  </si>
-  <si>
-    <t>Угол горизонтальный CPO 90 (50 х 50)</t>
-  </si>
-  <si>
-    <t>Уплотнительный модуль МКС 20/О 5-14мм</t>
-  </si>
-  <si>
-    <t>Уплотнительный модуль МКС 40/Ø 17-34 мм</t>
-  </si>
-  <si>
-    <t>Держатель проводника Rd8, DEHNGRIP NIRO h20 с отв.8мм М6</t>
-  </si>
-  <si>
-    <t>Диод КД209А ТТЗ.362.008 ТУ</t>
-  </si>
-  <si>
-    <t>Заглушка  25х25 для трубы профильной ПВД черная</t>
-  </si>
-  <si>
-    <t>Заглушка 10707 Legrand DPL 65х195</t>
-  </si>
-  <si>
-    <t>Кабель-канал 10453 Legrand DPL 195х65 (2м)</t>
-  </si>
-  <si>
-    <t>Компрессионный блок МКС КБ 120</t>
-  </si>
-  <si>
-    <t>Консоль с опорой ML 300мм (шт)</t>
-  </si>
-  <si>
-    <t>Коробка клеммная МТ Р307(-60+40) 2-6х20НК(А)-1х20НК(В)-6х20НК(С)-4х26(П) 1ЕхеLLCGbXT6, ip66</t>
-  </si>
-  <si>
-    <t>Коробка клеммная МТ Р402(-60+40)12-2х20НК(А)-2х20НК(С)-1,5х11(П), 1ЕхеLLCGbXT6, ip66, 110х75х55</t>
-  </si>
-  <si>
-    <t>Коробка клеммная МТ Р403(-60+40) 2-4х20НК(А)-4х20НК(С)-2,5х20(П),1ЕхеLLCGbXT6, ip66, 160х175х55</t>
-  </si>
-  <si>
-    <t>Коробка клеммная МТ Р407(-60+40) 2-8х20НК(А)-8х20НК(С)-2,5х31(П),1ЕхеLLCGbXT6, ip66, 220х120х90</t>
+    <t>Выключатель двухклавишный IP55</t>
+  </si>
+  <si>
+    <t>Геркон КЭМ-2</t>
+  </si>
+  <si>
+    <t>Держатель для полосы заземления К-188 У2 (цинк)</t>
+  </si>
+  <si>
+    <t>Угол горизонтальный CPO 90 (100 х 50)</t>
+  </si>
+  <si>
+    <t>Считыватель бесконтактный для proxi-карт, RD 26-REH-КМ АЯКС Ex mb IIC T5 Gb X , IP67</t>
+  </si>
+  <si>
+    <t>Считыватель бесконтактный для proxi-карт, Proxy-3МA IP20</t>
+  </si>
+  <si>
+    <t>Скоба металлическая СМО 16-17 49152 КВТ</t>
+  </si>
+  <si>
+    <t>Резьбовой крепежный элемент с наружной резьбой РКН-15 (ММРн-15)</t>
+  </si>
+  <si>
+    <t>Резьбовой крепежный элемент с внутренней резьбой Ркв-15</t>
+  </si>
+  <si>
+    <t>Профиль PSM (3000) арт. 34181</t>
   </si>
   <si>
     <t>Коробка клеммная МТ Р407(-60+40) 2-8х20НК(А)-8х20НК(С)-4х26(П),1ЕхеLLCGbXT6, ip66, 220х120х90</t>
@@ -576,60 +582,21 @@
     <t>Коробка распаячная КМ41242 IP55</t>
   </si>
   <si>
+    <t>Крышка Угол горизонтальный CPO 90 (100х50)</t>
+  </si>
+  <si>
+    <t>Крышка на Угол вертикальный внешний CD 90 (50 х 50)</t>
+  </si>
+  <si>
+    <t>Крышка (50х15х3000)</t>
+  </si>
+  <si>
+    <t>Крышка (100х15х3000)</t>
+  </si>
+  <si>
     <t>Крепление для труб ПВХ с защелкой, 16 мм</t>
   </si>
   <si>
-    <t>Крышка (100х15х3000)</t>
-  </si>
-  <si>
-    <t>Крышка (50х15х3000)</t>
-  </si>
-  <si>
-    <t>Крышка на Угол вертикальный внешний CD 90 (50 х 50)</t>
-  </si>
-  <si>
-    <t>Крышка Угол горизонтальный CPO 90 (100х50)</t>
-  </si>
-  <si>
-    <t>Профиль PSM (3000) арт. 34181</t>
-  </si>
-  <si>
-    <t>Резьбовой крепежный элемент с внутренней резьбой Ркв-15</t>
-  </si>
-  <si>
-    <t>Резьбовой крепежный элемент с наружной резьбой РКН-15 (ММРн-15)</t>
-  </si>
-  <si>
-    <t>Скоба металлическая СМО 16-17 49152 КВТ</t>
-  </si>
-  <si>
-    <t>Считыватель бесконтактный для proxi-карт, Proxy-3МA IP20</t>
-  </si>
-  <si>
-    <t>Считыватель бесконтактный для proxi-карт, RD 26-REH-КМ АЯКС Ex mb IIC T5 Gb X , IP67</t>
-  </si>
-  <si>
-    <t>Угол горизонтальный CPO 90 (100 х 50)</t>
-  </si>
-  <si>
-    <t>Выключатель двухклавишный IP55</t>
-  </si>
-  <si>
-    <t>Геркон КЭМ-2</t>
-  </si>
-  <si>
-    <t>Держатель для полосы заземления К-188 У2 (цинк)</t>
-  </si>
-  <si>
-    <t>Плата питания ПСМ.11.00.00.01-02</t>
-  </si>
-  <si>
-    <t>Плата печатная ПСМ.11.00.01.01-02</t>
-  </si>
-  <si>
-    <t>Пластина для заземления PTCE арт. 37501</t>
-  </si>
-  <si>
     <t>Очки защитные для токарей.О15.</t>
   </si>
   <si>
@@ -642,93 +609,57 @@
     <t>Пост аварийной сигнализации загазованности в/защ.ПАСВ1-П-75-1Ж1К-В1 (=24В, -60..+40С) 1ExsIICT6</t>
   </si>
   <si>
+    <t>Магнит МС3 ЦО 14,5/4 ТУ 3498-005-12591667-2014</t>
+  </si>
+  <si>
+    <t>Пружина №442 НТ.110.000.007.0</t>
+  </si>
+  <si>
+    <t>Пружина крышки НТ.200.004.003.0</t>
+  </si>
+  <si>
+    <t>Пружина №467 НТ.200.000.029.0</t>
+  </si>
+  <si>
     <t>Пружина НТ.3.02.00.00.002-01</t>
   </si>
   <si>
-    <t>Пружина №467 НТ.200.000.029.0</t>
-  </si>
-  <si>
-    <t>Пружина крышки НТ.200.004.003.0</t>
-  </si>
-  <si>
-    <t>Пружина №442 НТ.110.000.007.0</t>
-  </si>
-  <si>
-    <t>Магнит МС3 ЦО 14,5/4 ТУ 3498-005-12591667-2014</t>
+    <t>Грунт-эмаль Дюропокс ДТМ 80 (внутрянка)</t>
+  </si>
+  <si>
+    <t>Дверь левс доводчиком2000х1000мм(ВхШ) полотно RAL 9003(белый)/коробка(RAL 9003)(белый)с цепью</t>
+  </si>
+  <si>
+    <t>Клапан обратный поворотный КОП 80-40 УХЛ1 19лс53нж (исп. фл. 3)</t>
+  </si>
+  <si>
+    <t>Задвижка клиновая литая ЗКЛ 80-40 УХЛ1 30лс15нж, класс герм.А (ряд 2, исп.фл.3)</t>
+  </si>
+  <si>
+    <t>Легкосбрасываемое окнная конструкция 1200х1100 мм / ПВХ-профили морозост. исп, RAL 9003 белый</t>
+  </si>
+  <si>
+    <t>Задвижка клиновая литая ЗКЛ 50-40 УХЛ1 30С15нж, класс герм.А (ряд 2, исп.фл.3)</t>
   </si>
   <si>
     <t>Задвижка ЗКС 31лс77нж Ду 15 Ру 40 МПа (соединение муфтовое Rc 1/2)</t>
   </si>
   <si>
-    <t>Задвижка клиновая литая ЗКЛ 50-40 УХЛ1 30С15нж, класс герм.А (ряд 2, исп.фл.3)</t>
-  </si>
-  <si>
-    <t>Задвижка клиновая литая ЗКЛ 80-40 УХЛ1 30лс15нж, класс герм.А (ряд 2, исп.фл.3)</t>
-  </si>
-  <si>
-    <t>Клапан обратный поворотный КОП 80-40 УХЛ1 19лс53нж (исп. фл. 3)</t>
-  </si>
-  <si>
-    <t>Дверь левс доводчиком2000х1000мм(ВхШ) полотно RAL 9003(белый)/коробка(RAL 9003)(белый)с цепью</t>
-  </si>
-  <si>
-    <t>Легкосбрасываемое окнная конструкция 1200х1100 мм / ПВХ-профили морозост. исп, RAL 9003 белый</t>
-  </si>
-  <si>
-    <t>Грунт-эмаль Дюропокс ДТМ 80 (внутрянка)</t>
+    <t>Болт М8-6gх25.58.019 ГОСТ 7798-70</t>
+  </si>
+  <si>
+    <t>Гайка М10-6Н ГОСТ 5927-70 (размер под ключ S=17)</t>
+  </si>
+  <si>
+    <t>Гайка М10.5 019 ГОСТ 5927-70</t>
+  </si>
+  <si>
+    <t>Гайка М14х1,5 ГОСТ 15522-70</t>
   </si>
   <si>
     <t>Гайка М16-6Н.8.20.019 ГОСТ 15523-70</t>
   </si>
   <si>
-    <t>Гайка М14х1,5 ГОСТ 15522-70</t>
-  </si>
-  <si>
-    <t>Гайка М10.5 019 ГОСТ 5927-70</t>
-  </si>
-  <si>
-    <t>Гайка М10-6Н ГОСТ 5927-70 (размер под ключ S=17)</t>
-  </si>
-  <si>
-    <t>Болт М8-6gх25.58.019 ГОСТ 7798-70</t>
-  </si>
-  <si>
-    <t>Заглушка 219х8 ГОСТ 09Г2С 17379-2001</t>
-  </si>
-  <si>
-    <t>Переход 57х6-89х8 09Г2С ГОСТ 17378-2001</t>
-  </si>
-  <si>
-    <t>Переход 89х8-76х8 ст. 09Г2С ГОСТ 17378-01</t>
-  </si>
-  <si>
-    <t>Переход 114х8-89х8 Ст.09Г2С ГОСТ 17378-01</t>
-  </si>
-  <si>
-    <t>Переход 159х8-114х8 09Г2С ГОСТ 17378-01</t>
-  </si>
-  <si>
-    <t>Заглушка 89х8 ст.09Г2С ГОСТ 17379-2001</t>
-  </si>
-  <si>
-    <t>Заглушка 159х8 ст.09Г2С ГОСТ 17379-2001</t>
-  </si>
-  <si>
-    <t>Заглушка 76х8 ст.09Г2С ГОСТ 17379-2001</t>
-  </si>
-  <si>
-    <t>Уголок 50х50х3 ГОСТ 8509-93/09Г2С ГОСТ 19281-2014</t>
-  </si>
-  <si>
-    <t>Труба D57х6 ГОСТ 8732-78/ 09Г2С ГОСТ 4543-2016</t>
-  </si>
-  <si>
-    <t>Труба D219х8 ГОСТ 8732-78/ 09Г2С ГОСТ 8731-74</t>
-  </si>
-  <si>
-    <t>Круг D45 Ст.40Х ГОСТ 4543-71</t>
-  </si>
-  <si>
     <t>Лист чечевица В-К-ПУ-3,0 Ст.09Г2С ГОСТ 8568-77</t>
   </si>
   <si>
@@ -766,6 +697,33 @@
   </si>
   <si>
     <t>Кольцо уплотнительное НТ 202.003.004.0</t>
+  </si>
+  <si>
+    <t>Пластина WNMG 080408-GP GM3225 GESAC</t>
+  </si>
+  <si>
+    <t>Пластина CCMT09T308-GP GM3225 GESAC</t>
+  </si>
+  <si>
+    <t>Пластина SPGT060204-DG AT9030</t>
+  </si>
+  <si>
+    <t>Фреза концевая твердосплавная GE-D10.0-25L-4F-10D-75L</t>
+  </si>
+  <si>
+    <t>Пластина R390-11 T3 08M-PM 1130 SANDVIK (кратно12 для корпуса ПСМ, кратно 2 -для верх.корп.КМР)</t>
+  </si>
+  <si>
+    <t>Фреза концевая твердосплавная D5*HRC55*L100*25*4F</t>
+  </si>
+  <si>
+    <t>Винт М4х6 ГОСТ 17473-80</t>
+  </si>
+  <si>
+    <t>Болт М5х40 оцинк. ГОСТ 7805-70</t>
+  </si>
+  <si>
+    <t>Шайба 5.01.019 ГОСТ 11371-78</t>
   </si>
   <si>
     <t>Кольцо А75х1,7 ГОСТ 13943-86_</t>
@@ -1205,14 +1163,14 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr autoPageBreaks="0" fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F210"/>
+  <dimension ref="A1:F198"/>
   <sheetFormatPr defaultColWidth="10.5" defaultRowHeight="11.45" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="5.1640625" style="1" customWidth="1"/>
     <col min="2" max="2" width="46.6640625" style="1" customWidth="1"/>
     <col min="3" max="3" width="74.83203125" style="1" customWidth="1"/>
     <col min="4" max="4" width="14.1640625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="18.5" style="1" customWidth="1"/>
+    <col min="5" max="5" width="13" style="1" customWidth="1"/>
     <col min="6" max="6" width="14.5" style="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1260,16 +1218,16 @@
       </c>
       <c r="B3" s="4"/>
       <c r="C3" s="8" t="s">
-        <v>95</v>
+        <v>84</v>
       </c>
       <c r="D3" s="5">
-        <v>36.9</v>
+        <v>15</v>
       </c>
       <c r="E3" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="F3" s="4" t="s">
         <v>9</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1278,16 +1236,16 @@
       </c>
       <c r="B4" s="4"/>
       <c r="C4" s="8" t="s">
-        <v>96</v>
+        <v>85</v>
       </c>
       <c r="D4" s="5">
-        <v>3.6</v>
+        <v>9</v>
       </c>
       <c r="E4" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="F4" s="4" t="s">
         <v>9</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1296,16 +1254,16 @@
       </c>
       <c r="B5" s="4"/>
       <c r="C5" s="8" t="s">
-        <v>97</v>
+        <v>86</v>
       </c>
       <c r="D5" s="5">
-        <v>6.6</v>
+        <v>21</v>
       </c>
       <c r="E5" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="F5" s="4" t="s">
         <v>9</v>
-      </c>
-      <c r="F5" s="4" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1314,16 +1272,16 @@
       </c>
       <c r="B6" s="4"/>
       <c r="C6" s="8" t="s">
-        <v>98</v>
+        <v>87</v>
       </c>
       <c r="D6" s="5">
-        <v>0.33</v>
+        <v>60</v>
       </c>
       <c r="E6" s="6" t="s">
         <v>11</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1332,16 +1290,16 @@
       </c>
       <c r="B7" s="4"/>
       <c r="C7" s="8" t="s">
-        <v>99</v>
+        <v>88</v>
       </c>
       <c r="D7" s="5">
-        <v>0.15</v>
+        <v>6</v>
       </c>
       <c r="E7" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F7" s="4" t="s">
         <v>9</v>
-      </c>
-      <c r="F7" s="4" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1350,16 +1308,16 @@
       </c>
       <c r="B8" s="4"/>
       <c r="C8" s="8" t="s">
-        <v>100</v>
+        <v>89</v>
       </c>
       <c r="D8" s="5">
         <v>0.75</v>
       </c>
       <c r="E8" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F8" s="4" t="s">
         <v>9</v>
-      </c>
-      <c r="F8" s="4" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1368,16 +1326,16 @@
       </c>
       <c r="B9" s="4"/>
       <c r="C9" s="8" t="s">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="D9" s="5">
-        <v>52.05</v>
+        <v>5.4</v>
       </c>
       <c r="E9" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F9" s="4" t="s">
         <v>9</v>
-      </c>
-      <c r="F9" s="4" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1386,16 +1344,16 @@
       </c>
       <c r="B10" s="4"/>
       <c r="C10" s="8" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="D10" s="5">
-        <v>6</v>
+        <v>0.33</v>
       </c>
       <c r="E10" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="F10" s="4" t="s">
         <v>9</v>
-      </c>
-      <c r="F10" s="4" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1404,16 +1362,16 @@
       </c>
       <c r="B11" s="4"/>
       <c r="C11" s="8" t="s">
-        <v>103</v>
+        <v>92</v>
       </c>
       <c r="D11" s="5">
-        <v>60</v>
+        <v>0.15</v>
       </c>
       <c r="E11" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F11" s="4" t="s">
         <v>9</v>
-      </c>
-      <c r="F11" s="4" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1422,16 +1380,16 @@
       </c>
       <c r="B12" s="4"/>
       <c r="C12" s="8" t="s">
-        <v>104</v>
+        <v>93</v>
       </c>
       <c r="D12" s="5">
-        <v>5.4</v>
+        <v>6.6</v>
       </c>
       <c r="E12" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F12" s="4" t="s">
         <v>9</v>
-      </c>
-      <c r="F12" s="4" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1440,16 +1398,16 @@
       </c>
       <c r="B13" s="4"/>
       <c r="C13" s="8" t="s">
-        <v>105</v>
+        <v>94</v>
       </c>
       <c r="D13" s="5">
-        <v>0.09</v>
+        <v>3.6</v>
       </c>
       <c r="E13" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F13" s="4" t="s">
         <v>9</v>
-      </c>
-      <c r="F13" s="4" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1458,16 +1416,16 @@
       </c>
       <c r="B14" s="4"/>
       <c r="C14" s="8" t="s">
-        <v>106</v>
+        <v>95</v>
       </c>
       <c r="D14" s="5">
-        <v>15</v>
+        <v>36.9</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1476,16 +1434,16 @@
       </c>
       <c r="B15" s="4"/>
       <c r="C15" s="8" t="s">
-        <v>107</v>
+        <v>96</v>
       </c>
       <c r="D15" s="5">
-        <v>38.700000000000003</v>
+        <v>0.3</v>
       </c>
       <c r="E15" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F15" s="4" t="s">
         <v>9</v>
-      </c>
-      <c r="F15" s="4" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1494,16 +1452,16 @@
       </c>
       <c r="B16" s="4"/>
       <c r="C16" s="8" t="s">
-        <v>108</v>
+        <v>97</v>
       </c>
       <c r="D16" s="5">
-        <v>47.4</v>
+        <v>52.05</v>
       </c>
       <c r="E16" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F16" s="4" t="s">
         <v>9</v>
-      </c>
-      <c r="F16" s="4" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1512,16 +1470,16 @@
       </c>
       <c r="B17" s="4"/>
       <c r="C17" s="8" t="s">
-        <v>109</v>
+        <v>98</v>
       </c>
       <c r="D17" s="5">
         <v>90</v>
       </c>
       <c r="E17" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F17" s="4" t="s">
         <v>9</v>
-      </c>
-      <c r="F17" s="4" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1530,16 +1488,16 @@
       </c>
       <c r="B18" s="4"/>
       <c r="C18" s="8" t="s">
-        <v>110</v>
+        <v>99</v>
       </c>
       <c r="D18" s="5">
-        <v>15.9</v>
+        <v>47.4</v>
       </c>
       <c r="E18" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F18" s="4" t="s">
         <v>9</v>
-      </c>
-      <c r="F18" s="4" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="19" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1548,16 +1506,16 @@
       </c>
       <c r="B19" s="4"/>
       <c r="C19" s="8" t="s">
-        <v>111</v>
+        <v>100</v>
       </c>
       <c r="D19" s="5">
-        <v>472.8</v>
+        <v>15.9</v>
       </c>
       <c r="E19" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F19" s="4" t="s">
         <v>9</v>
-      </c>
-      <c r="F19" s="4" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="20" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1566,16 +1524,16 @@
       </c>
       <c r="B20" s="4"/>
       <c r="C20" s="8" t="s">
-        <v>112</v>
+        <v>101</v>
       </c>
       <c r="D20" s="5">
-        <v>112.8</v>
+        <v>472.8</v>
       </c>
       <c r="E20" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F20" s="4" t="s">
         <v>9</v>
-      </c>
-      <c r="F20" s="4" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="21" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1584,16 +1542,16 @@
       </c>
       <c r="B21" s="4"/>
       <c r="C21" s="8" t="s">
-        <v>12</v>
+        <v>102</v>
       </c>
       <c r="D21" s="5">
-        <v>28.2</v>
+        <v>112.8</v>
       </c>
       <c r="E21" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F21" s="4" t="s">
         <v>9</v>
-      </c>
-      <c r="F21" s="4" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="22" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1602,16 +1560,16 @@
       </c>
       <c r="B22" s="4"/>
       <c r="C22" s="8" t="s">
-        <v>113</v>
+        <v>13</v>
       </c>
       <c r="D22" s="5">
-        <v>20.7</v>
+        <v>28.2</v>
       </c>
       <c r="E22" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F22" s="4" t="s">
         <v>9</v>
-      </c>
-      <c r="F22" s="4" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="23" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1620,16 +1578,16 @@
       </c>
       <c r="B23" s="4"/>
       <c r="C23" s="8" t="s">
-        <v>114</v>
+        <v>103</v>
       </c>
       <c r="D23" s="5">
-        <v>0.3</v>
+        <v>20.7</v>
       </c>
       <c r="E23" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F23" s="4" t="s">
         <v>9</v>
-      </c>
-      <c r="F23" s="4" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="24" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1638,16 +1596,16 @@
       </c>
       <c r="B24" s="4"/>
       <c r="C24" s="8" t="s">
-        <v>115</v>
+        <v>104</v>
       </c>
       <c r="D24" s="5">
-        <v>1.05</v>
+        <v>22.5</v>
       </c>
       <c r="E24" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F24" s="4" t="s">
         <v>9</v>
-      </c>
-      <c r="F24" s="4" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="25" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1656,16 +1614,16 @@
       </c>
       <c r="B25" s="4"/>
       <c r="C25" s="8" t="s">
-        <v>116</v>
+        <v>105</v>
       </c>
       <c r="D25" s="5">
-        <v>20.7</v>
+        <v>13.65</v>
       </c>
       <c r="E25" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F25" s="4" t="s">
         <v>9</v>
-      </c>
-      <c r="F25" s="4" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="26" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1674,16 +1632,16 @@
       </c>
       <c r="B26" s="4"/>
       <c r="C26" s="8" t="s">
-        <v>117</v>
+        <v>106</v>
       </c>
       <c r="D26" s="5">
-        <v>33.15</v>
+        <v>21.9</v>
       </c>
       <c r="E26" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F26" s="4" t="s">
         <v>9</v>
-      </c>
-      <c r="F26" s="4" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="27" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1692,16 +1650,16 @@
       </c>
       <c r="B27" s="4"/>
       <c r="C27" s="8" t="s">
-        <v>118</v>
+        <v>107</v>
       </c>
       <c r="D27" s="5">
+        <v>6.6</v>
+      </c>
+      <c r="E27" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F27" s="4" t="s">
         <v>9</v>
-      </c>
-      <c r="E27" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="F27" s="4" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="28" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1710,16 +1668,16 @@
       </c>
       <c r="B28" s="4"/>
       <c r="C28" s="8" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="D28" s="5">
-        <v>21</v>
+        <v>0.09</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="29" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1728,16 +1686,16 @@
       </c>
       <c r="B29" s="4"/>
       <c r="C29" s="8" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="D29" s="5">
-        <v>40.5</v>
+        <v>55.8</v>
       </c>
       <c r="E29" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F29" s="4" t="s">
         <v>9</v>
-      </c>
-      <c r="F29" s="4" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="30" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1746,16 +1704,16 @@
       </c>
       <c r="B30" s="4"/>
       <c r="C30" s="8" t="s">
-        <v>121</v>
+        <v>110</v>
       </c>
       <c r="D30" s="5">
         <v>20.399999999999999</v>
       </c>
       <c r="E30" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F30" s="4" t="s">
         <v>9</v>
-      </c>
-      <c r="F30" s="4" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="31" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1764,16 +1722,16 @@
       </c>
       <c r="B31" s="4"/>
       <c r="C31" s="8" t="s">
-        <v>122</v>
+        <v>111</v>
       </c>
       <c r="D31" s="5">
-        <v>55.8</v>
+        <v>40.5</v>
       </c>
       <c r="E31" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F31" s="4" t="s">
         <v>9</v>
-      </c>
-      <c r="F31" s="4" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="32" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1782,16 +1740,16 @@
       </c>
       <c r="B32" s="4"/>
       <c r="C32" s="8" t="s">
-        <v>123</v>
+        <v>112</v>
       </c>
       <c r="D32" s="5">
-        <v>6.6</v>
+        <v>33.15</v>
       </c>
       <c r="E32" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F32" s="4" t="s">
         <v>9</v>
-      </c>
-      <c r="F32" s="4" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="33" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1800,16 +1758,16 @@
       </c>
       <c r="B33" s="4"/>
       <c r="C33" s="8" t="s">
-        <v>124</v>
+        <v>113</v>
       </c>
       <c r="D33" s="5">
-        <v>21.9</v>
+        <v>20.7</v>
       </c>
       <c r="E33" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F33" s="4" t="s">
         <v>9</v>
-      </c>
-      <c r="F33" s="4" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="34" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1818,16 +1776,16 @@
       </c>
       <c r="B34" s="4"/>
       <c r="C34" s="8" t="s">
-        <v>125</v>
+        <v>114</v>
       </c>
       <c r="D34" s="5">
-        <v>13.65</v>
+        <v>38.700000000000003</v>
       </c>
       <c r="E34" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F34" s="4" t="s">
         <v>9</v>
-      </c>
-      <c r="F34" s="4" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="35" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1836,16 +1794,16 @@
       </c>
       <c r="B35" s="4"/>
       <c r="C35" s="8" t="s">
-        <v>126</v>
+        <v>115</v>
       </c>
       <c r="D35" s="5">
-        <v>22.5</v>
+        <v>1.05</v>
       </c>
       <c r="E35" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F35" s="4" t="s">
         <v>9</v>
-      </c>
-      <c r="F35" s="4" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="36" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1890,7 +1848,7 @@
       </c>
       <c r="B38" s="4"/>
       <c r="C38" s="8" t="s">
-        <v>127</v>
+        <v>116</v>
       </c>
       <c r="D38" s="5">
         <v>200</v>
@@ -1908,7 +1866,7 @@
       </c>
       <c r="B39" s="4"/>
       <c r="C39" s="8" t="s">
-        <v>128</v>
+        <v>117</v>
       </c>
       <c r="D39" s="5">
         <v>200</v>
@@ -1926,7 +1884,7 @@
       </c>
       <c r="B40" s="4"/>
       <c r="C40" s="8" t="s">
-        <v>129</v>
+        <v>118</v>
       </c>
       <c r="D40" s="5">
         <v>200</v>
@@ -1944,7 +1902,7 @@
       </c>
       <c r="B41" s="4"/>
       <c r="C41" s="8" t="s">
-        <v>130</v>
+        <v>119</v>
       </c>
       <c r="D41" s="5">
         <v>200</v>
@@ -1962,7 +1920,7 @@
       </c>
       <c r="B42" s="4"/>
       <c r="C42" s="8" t="s">
-        <v>131</v>
+        <v>120</v>
       </c>
       <c r="D42" s="5">
         <v>200</v>
@@ -1980,7 +1938,7 @@
       </c>
       <c r="B43" s="4"/>
       <c r="C43" s="8" t="s">
-        <v>132</v>
+        <v>121</v>
       </c>
       <c r="D43" s="5">
         <v>200</v>
@@ -1998,7 +1956,7 @@
       </c>
       <c r="B44" s="4"/>
       <c r="C44" s="8" t="s">
-        <v>133</v>
+        <v>122</v>
       </c>
       <c r="D44" s="5">
         <v>1</v>
@@ -2055,7 +2013,7 @@
         <v>23</v>
       </c>
       <c r="D47" s="5">
-        <v>42</v>
+        <v>153</v>
       </c>
       <c r="E47" s="6" t="s">
         <v>7</v>
@@ -2070,10 +2028,10 @@
       </c>
       <c r="B48" s="4"/>
       <c r="C48" s="8" t="s">
-        <v>134</v>
+        <v>25</v>
       </c>
       <c r="D48" s="5">
-        <v>8</v>
+        <v>42</v>
       </c>
       <c r="E48" s="6" t="s">
         <v>7</v>
@@ -2088,10 +2046,10 @@
       </c>
       <c r="B49" s="4"/>
       <c r="C49" s="8" t="s">
-        <v>135</v>
+        <v>123</v>
       </c>
       <c r="D49" s="5">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E49" s="6" t="s">
         <v>7</v>
@@ -2106,10 +2064,10 @@
       </c>
       <c r="B50" s="4"/>
       <c r="C50" s="8" t="s">
-        <v>136</v>
+        <v>124</v>
       </c>
       <c r="D50" s="5">
-        <v>64</v>
+        <v>5</v>
       </c>
       <c r="E50" s="6" t="s">
         <v>7</v>
@@ -2124,10 +2082,10 @@
       </c>
       <c r="B51" s="4"/>
       <c r="C51" s="8" t="s">
-        <v>137</v>
+        <v>125</v>
       </c>
       <c r="D51" s="5">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="E51" s="6" t="s">
         <v>7</v>
@@ -2142,10 +2100,10 @@
       </c>
       <c r="B52" s="4"/>
       <c r="C52" s="8" t="s">
-        <v>138</v>
+        <v>126</v>
       </c>
       <c r="D52" s="5">
-        <v>144</v>
+        <v>57</v>
       </c>
       <c r="E52" s="6" t="s">
         <v>7</v>
@@ -2160,10 +2118,10 @@
       </c>
       <c r="B53" s="4"/>
       <c r="C53" s="8" t="s">
-        <v>139</v>
+        <v>127</v>
       </c>
       <c r="D53" s="5">
-        <v>8</v>
+        <v>144</v>
       </c>
       <c r="E53" s="6" t="s">
         <v>7</v>
@@ -2178,10 +2136,10 @@
       </c>
       <c r="B54" s="4"/>
       <c r="C54" s="8" t="s">
-        <v>140</v>
+        <v>26</v>
       </c>
       <c r="D54" s="5">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E54" s="6" t="s">
         <v>7</v>
@@ -2196,7 +2154,7 @@
       </c>
       <c r="B55" s="4"/>
       <c r="C55" s="8" t="s">
-        <v>141</v>
+        <v>128</v>
       </c>
       <c r="D55" s="5">
         <v>8</v>
@@ -2214,7 +2172,7 @@
       </c>
       <c r="B56" s="4"/>
       <c r="C56" s="8" t="s">
-        <v>142</v>
+        <v>129</v>
       </c>
       <c r="D56" s="5">
         <v>8</v>
@@ -2232,10 +2190,10 @@
       </c>
       <c r="B57" s="4"/>
       <c r="C57" s="8" t="s">
-        <v>143</v>
+        <v>130</v>
       </c>
       <c r="D57" s="5">
-        <v>56</v>
+        <v>8</v>
       </c>
       <c r="E57" s="6" t="s">
         <v>7</v>
@@ -2250,13 +2208,13 @@
       </c>
       <c r="B58" s="4"/>
       <c r="C58" s="8" t="s">
-        <v>144</v>
+        <v>131</v>
       </c>
       <c r="D58" s="5">
-        <v>40</v>
+        <v>8</v>
       </c>
       <c r="E58" s="6" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="F58" s="4" t="s">
         <v>24</v>
@@ -2268,13 +2226,13 @@
       </c>
       <c r="B59" s="4"/>
       <c r="C59" s="8" t="s">
-        <v>145</v>
+        <v>132</v>
       </c>
       <c r="D59" s="5">
-        <v>320</v>
+        <v>56</v>
       </c>
       <c r="E59" s="6" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="F59" s="4" t="s">
         <v>24</v>
@@ -2286,13 +2244,13 @@
       </c>
       <c r="B60" s="4"/>
       <c r="C60" s="8" t="s">
-        <v>146</v>
+        <v>133</v>
       </c>
       <c r="D60" s="5">
-        <v>100.8</v>
+        <v>200</v>
       </c>
       <c r="E60" s="6" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="F60" s="4" t="s">
         <v>24</v>
@@ -2304,13 +2262,13 @@
       </c>
       <c r="B61" s="4"/>
       <c r="C61" s="8" t="s">
-        <v>147</v>
-      </c>
-      <c r="D61" s="7">
-        <v>1199</v>
+        <v>134</v>
+      </c>
+      <c r="D61" s="5">
+        <v>8</v>
       </c>
       <c r="E61" s="6" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="F61" s="4" t="s">
         <v>24</v>
@@ -2322,13 +2280,13 @@
       </c>
       <c r="B62" s="4"/>
       <c r="C62" s="8" t="s">
-        <v>148</v>
+        <v>135</v>
       </c>
       <c r="D62" s="5">
-        <v>56</v>
+        <v>8</v>
       </c>
       <c r="E62" s="6" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="F62" s="4" t="s">
         <v>24</v>
@@ -2340,13 +2298,13 @@
       </c>
       <c r="B63" s="4"/>
       <c r="C63" s="8" t="s">
-        <v>149</v>
+        <v>27</v>
       </c>
       <c r="D63" s="5">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E63" s="6" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="F63" s="4" t="s">
         <v>24</v>
@@ -2358,13 +2316,13 @@
       </c>
       <c r="B64" s="4"/>
       <c r="C64" s="8" t="s">
-        <v>150</v>
+        <v>28</v>
       </c>
       <c r="D64" s="5">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="E64" s="6" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F64" s="4" t="s">
         <v>24</v>
@@ -2376,13 +2334,13 @@
       </c>
       <c r="B65" s="4"/>
       <c r="C65" s="8" t="s">
-        <v>151</v>
+        <v>136</v>
       </c>
       <c r="D65" s="5">
-        <v>861.2</v>
+        <v>64</v>
       </c>
       <c r="E65" s="6" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="F65" s="4" t="s">
         <v>24</v>
@@ -2394,13 +2352,13 @@
       </c>
       <c r="B66" s="4"/>
       <c r="C66" s="8" t="s">
-        <v>152</v>
+        <v>137</v>
       </c>
       <c r="D66" s="5">
-        <v>98</v>
+        <v>240</v>
       </c>
       <c r="E66" s="6" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="F66" s="4" t="s">
         <v>24</v>
@@ -2412,13 +2370,13 @@
       </c>
       <c r="B67" s="4"/>
       <c r="C67" s="8" t="s">
-        <v>153</v>
+        <v>138</v>
       </c>
       <c r="D67" s="5">
-        <v>288</v>
+        <v>48</v>
       </c>
       <c r="E67" s="6" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="F67" s="4" t="s">
         <v>24</v>
@@ -2430,13 +2388,13 @@
       </c>
       <c r="B68" s="4"/>
       <c r="C68" s="8" t="s">
-        <v>154</v>
+        <v>139</v>
       </c>
       <c r="D68" s="5">
-        <v>989</v>
+        <v>40</v>
       </c>
       <c r="E68" s="6" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F68" s="4" t="s">
         <v>24</v>
@@ -2448,13 +2406,13 @@
       </c>
       <c r="B69" s="4"/>
       <c r="C69" s="8" t="s">
-        <v>155</v>
+        <v>140</v>
       </c>
       <c r="D69" s="5">
-        <v>396.5</v>
+        <v>88</v>
       </c>
       <c r="E69" s="6" t="s">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="F69" s="4" t="s">
         <v>24</v>
@@ -2466,13 +2424,13 @@
       </c>
       <c r="B70" s="4"/>
       <c r="C70" s="8" t="s">
-        <v>156</v>
+        <v>30</v>
       </c>
       <c r="D70" s="5">
-        <v>0.6</v>
+        <v>3</v>
       </c>
       <c r="E70" s="6" t="s">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="F70" s="4" t="s">
         <v>24</v>
@@ -2484,13 +2442,13 @@
       </c>
       <c r="B71" s="4"/>
       <c r="C71" s="8" t="s">
-        <v>157</v>
+        <v>141</v>
       </c>
       <c r="D71" s="5">
-        <v>16</v>
+        <v>560</v>
       </c>
       <c r="E71" s="6" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="F71" s="4" t="s">
         <v>24</v>
@@ -2502,13 +2460,13 @@
       </c>
       <c r="B72" s="4"/>
       <c r="C72" s="8" t="s">
-        <v>158</v>
+        <v>142</v>
       </c>
       <c r="D72" s="5">
-        <v>274.8</v>
+        <v>192</v>
       </c>
       <c r="E72" s="6" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="F72" s="4" t="s">
         <v>24</v>
@@ -2520,13 +2478,13 @@
       </c>
       <c r="B73" s="4"/>
       <c r="C73" s="8" t="s">
-        <v>159</v>
+        <v>143</v>
       </c>
       <c r="D73" s="5">
-        <v>48</v>
+        <v>76</v>
       </c>
       <c r="E73" s="6" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="F73" s="4" t="s">
         <v>24</v>
@@ -2538,13 +2496,13 @@
       </c>
       <c r="B74" s="4"/>
       <c r="C74" s="8" t="s">
-        <v>160</v>
+        <v>144</v>
       </c>
       <c r="D74" s="5">
-        <v>259</v>
+        <v>10</v>
       </c>
       <c r="E74" s="6" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="F74" s="4" t="s">
         <v>24</v>
@@ -2556,13 +2514,13 @@
       </c>
       <c r="B75" s="4"/>
       <c r="C75" s="8" t="s">
-        <v>161</v>
-      </c>
-      <c r="D75" s="7">
-        <v>1040</v>
+        <v>145</v>
+      </c>
+      <c r="D75" s="5">
+        <v>16.8</v>
       </c>
       <c r="E75" s="6" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F75" s="4" t="s">
         <v>24</v>
@@ -2574,13 +2532,13 @@
       </c>
       <c r="B76" s="4"/>
       <c r="C76" s="8" t="s">
-        <v>119</v>
+        <v>146</v>
       </c>
       <c r="D76" s="5">
-        <v>602.20000000000005</v>
+        <v>48</v>
       </c>
       <c r="E76" s="6" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="F76" s="4" t="s">
         <v>24</v>
@@ -2592,10 +2550,10 @@
       </c>
       <c r="B77" s="4"/>
       <c r="C77" s="8" t="s">
-        <v>25</v>
+        <v>147</v>
       </c>
       <c r="D77" s="5">
-        <v>6</v>
+        <v>32</v>
       </c>
       <c r="E77" s="6" t="s">
         <v>7</v>
@@ -2610,13 +2568,13 @@
       </c>
       <c r="B78" s="4"/>
       <c r="C78" s="8" t="s">
-        <v>26</v>
+        <v>148</v>
       </c>
       <c r="D78" s="5">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="E78" s="6" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="F78" s="4" t="s">
         <v>24</v>
@@ -2628,13 +2586,13 @@
       </c>
       <c r="B79" s="4"/>
       <c r="C79" s="8" t="s">
-        <v>162</v>
+        <v>149</v>
       </c>
       <c r="D79" s="5">
-        <v>40</v>
+        <v>16</v>
       </c>
       <c r="E79" s="6" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="F79" s="4" t="s">
         <v>24</v>
@@ -2646,10 +2604,10 @@
       </c>
       <c r="B80" s="4"/>
       <c r="C80" s="8" t="s">
-        <v>163</v>
+        <v>150</v>
       </c>
       <c r="D80" s="5">
-        <v>32</v>
+        <v>112</v>
       </c>
       <c r="E80" s="6" t="s">
         <v>7</v>
@@ -2658,73 +2616,73 @@
         <v>24</v>
       </c>
     </row>
-    <row r="81" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A81" s="3">
         <v>80</v>
       </c>
       <c r="B81" s="4"/>
       <c r="C81" s="8" t="s">
-        <v>164</v>
+        <v>151</v>
       </c>
       <c r="D81" s="5">
-        <v>88</v>
+        <v>18</v>
       </c>
       <c r="E81" s="6" t="s">
-        <v>27</v>
+        <v>7</v>
       </c>
       <c r="F81" s="4" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="82" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A82" s="3">
         <v>81</v>
       </c>
       <c r="B82" s="4"/>
       <c r="C82" s="8" t="s">
-        <v>28</v>
+        <v>152</v>
       </c>
       <c r="D82" s="5">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E82" s="6" t="s">
-        <v>29</v>
+        <v>7</v>
       </c>
       <c r="F82" s="4" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="83" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A83" s="3">
         <v>82</v>
       </c>
       <c r="B83" s="4"/>
       <c r="C83" s="8" t="s">
-        <v>165</v>
+        <v>153</v>
       </c>
       <c r="D83" s="5">
-        <v>16.8</v>
+        <v>10</v>
       </c>
       <c r="E83" s="6" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="F83" s="4" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="84" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A84" s="3">
         <v>83</v>
       </c>
       <c r="B84" s="4"/>
       <c r="C84" s="8" t="s">
-        <v>166</v>
+        <v>154</v>
       </c>
       <c r="D84" s="5">
-        <v>48</v>
+        <v>10</v>
       </c>
       <c r="E84" s="6" t="s">
-        <v>30</v>
+        <v>7</v>
       </c>
       <c r="F84" s="4" t="s">
         <v>24</v>
@@ -2736,13 +2694,13 @@
       </c>
       <c r="B85" s="4"/>
       <c r="C85" s="8" t="s">
-        <v>167</v>
+        <v>155</v>
       </c>
       <c r="D85" s="5">
-        <v>64</v>
+        <v>40</v>
       </c>
       <c r="E85" s="6" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F85" s="4" t="s">
         <v>24</v>
@@ -2754,13 +2712,13 @@
       </c>
       <c r="B86" s="4"/>
       <c r="C86" s="8" t="s">
-        <v>31</v>
+        <v>156</v>
       </c>
       <c r="D86" s="5">
-        <v>160</v>
+        <v>320</v>
       </c>
       <c r="E86" s="6" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F86" s="4" t="s">
         <v>24</v>
@@ -2772,13 +2730,13 @@
       </c>
       <c r="B87" s="4"/>
       <c r="C87" s="8" t="s">
-        <v>32</v>
+        <v>157</v>
       </c>
       <c r="D87" s="5">
-        <v>6</v>
+        <v>100.8</v>
       </c>
       <c r="E87" s="6" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F87" s="4" t="s">
         <v>24</v>
@@ -2790,13 +2748,13 @@
       </c>
       <c r="B88" s="4"/>
       <c r="C88" s="8" t="s">
-        <v>168</v>
-      </c>
-      <c r="D88" s="5">
-        <v>240</v>
+        <v>158</v>
+      </c>
+      <c r="D88" s="7">
+        <v>1199</v>
       </c>
       <c r="E88" s="6" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F88" s="4" t="s">
         <v>24</v>
@@ -2808,13 +2766,13 @@
       </c>
       <c r="B89" s="4"/>
       <c r="C89" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="D89" s="5">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="E89" s="6" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F89" s="4" t="s">
         <v>24</v>
@@ -2826,13 +2784,13 @@
       </c>
       <c r="B90" s="4"/>
       <c r="C90" s="8" t="s">
-        <v>170</v>
+        <v>160</v>
       </c>
       <c r="D90" s="5">
-        <v>560</v>
+        <v>10</v>
       </c>
       <c r="E90" s="6" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F90" s="4" t="s">
         <v>24</v>
@@ -2844,13 +2802,13 @@
       </c>
       <c r="B91" s="4"/>
       <c r="C91" s="8" t="s">
-        <v>171</v>
+        <v>161</v>
       </c>
       <c r="D91" s="5">
-        <v>192</v>
+        <v>30</v>
       </c>
       <c r="E91" s="6" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F91" s="4" t="s">
         <v>24</v>
@@ -2862,13 +2820,13 @@
       </c>
       <c r="B92" s="4"/>
       <c r="C92" s="8" t="s">
-        <v>172</v>
+        <v>162</v>
       </c>
       <c r="D92" s="5">
-        <v>76</v>
+        <v>861.2</v>
       </c>
       <c r="E92" s="6" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F92" s="4" t="s">
         <v>24</v>
@@ -2880,13 +2838,13 @@
       </c>
       <c r="B93" s="4"/>
       <c r="C93" s="8" t="s">
-        <v>173</v>
+        <v>163</v>
       </c>
       <c r="D93" s="5">
+        <v>98</v>
+      </c>
+      <c r="E93" s="6" t="s">
         <v>10</v>
-      </c>
-      <c r="E93" s="6" t="s">
-        <v>7</v>
       </c>
       <c r="F93" s="4" t="s">
         <v>24</v>
@@ -2898,13 +2856,13 @@
       </c>
       <c r="B94" s="4"/>
       <c r="C94" s="8" t="s">
-        <v>174</v>
+        <v>164</v>
       </c>
       <c r="D94" s="5">
-        <v>40</v>
+        <v>288</v>
       </c>
       <c r="E94" s="6" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F94" s="4" t="s">
         <v>24</v>
@@ -2916,13 +2874,13 @@
       </c>
       <c r="B95" s="4"/>
       <c r="C95" s="8" t="s">
-        <v>175</v>
+        <v>165</v>
       </c>
       <c r="D95" s="5">
-        <v>16</v>
+        <v>989</v>
       </c>
       <c r="E95" s="6" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F95" s="4" t="s">
         <v>24</v>
@@ -2934,103 +2892,103 @@
       </c>
       <c r="B96" s="4"/>
       <c r="C96" s="8" t="s">
-        <v>176</v>
+        <v>166</v>
       </c>
       <c r="D96" s="5">
-        <v>112</v>
+        <v>396.5</v>
       </c>
       <c r="E96" s="6" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F96" s="4" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="97" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A97" s="3">
         <v>96</v>
       </c>
       <c r="B97" s="4"/>
       <c r="C97" s="8" t="s">
-        <v>177</v>
+        <v>167</v>
       </c>
       <c r="D97" s="5">
-        <v>18</v>
+        <v>0.6</v>
       </c>
       <c r="E97" s="6" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F97" s="4" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="98" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A98" s="3">
         <v>97</v>
       </c>
       <c r="B98" s="4"/>
       <c r="C98" s="8" t="s">
-        <v>178</v>
+        <v>168</v>
       </c>
       <c r="D98" s="5">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="E98" s="6" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F98" s="4" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="99" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A99" s="3">
         <v>98</v>
       </c>
       <c r="B99" s="4"/>
       <c r="C99" s="8" t="s">
-        <v>179</v>
+        <v>169</v>
       </c>
       <c r="D99" s="5">
+        <v>274.8</v>
+      </c>
+      <c r="E99" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="E99" s="6" t="s">
-        <v>7</v>
-      </c>
       <c r="F99" s="4" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="100" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A100" s="3">
         <v>99</v>
       </c>
       <c r="B100" s="4"/>
       <c r="C100" s="8" t="s">
-        <v>180</v>
+        <v>170</v>
       </c>
       <c r="D100" s="5">
+        <v>48</v>
+      </c>
+      <c r="E100" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="E100" s="6" t="s">
-        <v>7</v>
-      </c>
       <c r="F100" s="4" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="101" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A101" s="3">
         <v>100</v>
       </c>
       <c r="B101" s="4"/>
       <c r="C101" s="8" t="s">
-        <v>181</v>
+        <v>171</v>
       </c>
       <c r="D101" s="5">
-        <v>5</v>
+        <v>259</v>
       </c>
       <c r="E101" s="6" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F101" s="4" t="s">
         <v>24</v>
@@ -3042,13 +3000,13 @@
       </c>
       <c r="B102" s="4"/>
       <c r="C102" s="8" t="s">
-        <v>182</v>
-      </c>
-      <c r="D102" s="5">
-        <v>8</v>
+        <v>172</v>
+      </c>
+      <c r="D102" s="7">
+        <v>1040</v>
       </c>
       <c r="E102" s="6" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F102" s="4" t="s">
         <v>24</v>
@@ -3060,28 +3018,28 @@
       </c>
       <c r="B103" s="4"/>
       <c r="C103" s="8" t="s">
-        <v>183</v>
+        <v>86</v>
       </c>
       <c r="D103" s="5">
-        <v>75</v>
+        <v>602.20000000000005</v>
       </c>
       <c r="E103" s="6" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F103" s="4" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="104" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A104" s="3">
         <v>103</v>
       </c>
       <c r="B104" s="4"/>
       <c r="C104" s="8" t="s">
-        <v>184</v>
+        <v>33</v>
       </c>
       <c r="D104" s="5">
-        <v>57</v>
+        <v>24</v>
       </c>
       <c r="E104" s="6" t="s">
         <v>7</v>
@@ -3096,10 +3054,10 @@
       </c>
       <c r="B105" s="4"/>
       <c r="C105" s="8" t="s">
-        <v>185</v>
+        <v>173</v>
       </c>
       <c r="D105" s="5">
-        <v>144</v>
+        <v>8</v>
       </c>
       <c r="E105" s="6" t="s">
         <v>7</v>
@@ -3114,10 +3072,10 @@
       </c>
       <c r="B106" s="4"/>
       <c r="C106" s="8" t="s">
-        <v>186</v>
+        <v>174</v>
       </c>
       <c r="D106" s="5">
-        <v>32</v>
+        <v>112</v>
       </c>
       <c r="E106" s="6" t="s">
         <v>7</v>
@@ -3132,10 +3090,10 @@
       </c>
       <c r="B107" s="4"/>
       <c r="C107" s="8" t="s">
-        <v>187</v>
+        <v>175</v>
       </c>
       <c r="D107" s="5">
-        <v>32</v>
+        <v>400</v>
       </c>
       <c r="E107" s="6" t="s">
         <v>7</v>
@@ -3150,10 +3108,10 @@
       </c>
       <c r="B108" s="4"/>
       <c r="C108" s="8" t="s">
-        <v>188</v>
+        <v>34</v>
       </c>
       <c r="D108" s="5">
-        <v>40</v>
+        <v>160</v>
       </c>
       <c r="E108" s="6" t="s">
         <v>7</v>
@@ -3168,10 +3126,10 @@
       </c>
       <c r="B109" s="4"/>
       <c r="C109" s="8" t="s">
-        <v>189</v>
+        <v>176</v>
       </c>
       <c r="D109" s="5">
-        <v>298</v>
+        <v>32</v>
       </c>
       <c r="E109" s="6" t="s">
         <v>7</v>
@@ -3180,16 +3138,16 @@
         <v>24</v>
       </c>
     </row>
-    <row r="110" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A110" s="3">
         <v>109</v>
       </c>
       <c r="B110" s="4"/>
       <c r="C110" s="8" t="s">
-        <v>190</v>
+        <v>177</v>
       </c>
       <c r="D110" s="5">
-        <v>422</v>
+        <v>8</v>
       </c>
       <c r="E110" s="6" t="s">
         <v>7</v>
@@ -3204,10 +3162,10 @@
       </c>
       <c r="B111" s="4"/>
       <c r="C111" s="8" t="s">
-        <v>191</v>
+        <v>178</v>
       </c>
       <c r="D111" s="5">
-        <v>900</v>
+        <v>8</v>
       </c>
       <c r="E111" s="6" t="s">
         <v>7</v>
@@ -3222,10 +3180,10 @@
       </c>
       <c r="B112" s="4"/>
       <c r="C112" s="8" t="s">
-        <v>192</v>
+        <v>179</v>
       </c>
       <c r="D112" s="5">
-        <v>8</v>
+        <v>900</v>
       </c>
       <c r="E112" s="6" t="s">
         <v>7</v>
@@ -3234,16 +3192,16 @@
         <v>24</v>
       </c>
     </row>
-    <row r="113" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A113" s="3">
         <v>112</v>
       </c>
       <c r="B113" s="4"/>
       <c r="C113" s="8" t="s">
-        <v>193</v>
+        <v>180</v>
       </c>
       <c r="D113" s="5">
-        <v>8</v>
+        <v>422</v>
       </c>
       <c r="E113" s="6" t="s">
         <v>7</v>
@@ -3258,10 +3216,10 @@
       </c>
       <c r="B114" s="4"/>
       <c r="C114" s="8" t="s">
-        <v>194</v>
+        <v>181</v>
       </c>
       <c r="D114" s="5">
-        <v>32</v>
+        <v>298</v>
       </c>
       <c r="E114" s="6" t="s">
         <v>7</v>
@@ -3276,10 +3234,10 @@
       </c>
       <c r="B115" s="4"/>
       <c r="C115" s="8" t="s">
-        <v>195</v>
+        <v>182</v>
       </c>
       <c r="D115" s="5">
-        <v>8</v>
+        <v>40</v>
       </c>
       <c r="E115" s="6" t="s">
         <v>7</v>
@@ -3288,16 +3246,16 @@
         <v>24</v>
       </c>
     </row>
-    <row r="116" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A116" s="3">
         <v>115</v>
       </c>
       <c r="B116" s="4"/>
       <c r="C116" s="8" t="s">
-        <v>196</v>
+        <v>183</v>
       </c>
       <c r="D116" s="5">
-        <v>112</v>
+        <v>5</v>
       </c>
       <c r="E116" s="6" t="s">
         <v>7</v>
@@ -3312,10 +3270,10 @@
       </c>
       <c r="B117" s="4"/>
       <c r="C117" s="8" t="s">
-        <v>197</v>
+        <v>184</v>
       </c>
       <c r="D117" s="5">
-        <v>400</v>
+        <v>8</v>
       </c>
       <c r="E117" s="6" t="s">
         <v>7</v>
@@ -3324,16 +3282,16 @@
         <v>24</v>
       </c>
     </row>
-    <row r="118" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A118" s="3">
         <v>117</v>
       </c>
       <c r="B118" s="4"/>
       <c r="C118" s="8" t="s">
-        <v>33</v>
+        <v>185</v>
       </c>
       <c r="D118" s="5">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="E118" s="6" t="s">
         <v>7</v>
@@ -3348,10 +3306,10 @@
       </c>
       <c r="B119" s="4"/>
       <c r="C119" s="8" t="s">
-        <v>34</v>
+        <v>186</v>
       </c>
       <c r="D119" s="5">
-        <v>153</v>
+        <v>32</v>
       </c>
       <c r="E119" s="6" t="s">
         <v>7</v>
@@ -3366,10 +3324,10 @@
       </c>
       <c r="B120" s="4"/>
       <c r="C120" s="8" t="s">
-        <v>198</v>
+        <v>187</v>
       </c>
       <c r="D120" s="5">
-        <v>8</v>
+        <v>144</v>
       </c>
       <c r="E120" s="6" t="s">
         <v>7</v>
@@ -3384,10 +3342,10 @@
       </c>
       <c r="B121" s="4"/>
       <c r="C121" s="8" t="s">
-        <v>199</v>
+        <v>188</v>
       </c>
       <c r="D121" s="5">
-        <v>8</v>
+        <v>57</v>
       </c>
       <c r="E121" s="6" t="s">
         <v>7</v>
@@ -3402,10 +3360,10 @@
       </c>
       <c r="B122" s="4"/>
       <c r="C122" s="8" t="s">
-        <v>200</v>
+        <v>189</v>
       </c>
       <c r="D122" s="5">
-        <v>200</v>
+        <v>75</v>
       </c>
       <c r="E122" s="6" t="s">
         <v>7</v>
@@ -3423,10 +3381,10 @@
         <v>35</v>
       </c>
       <c r="D123" s="5">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="E123" s="6" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="F123" s="4" t="s">
         <v>36</v>
@@ -3438,13 +3396,13 @@
       </c>
       <c r="B124" s="4"/>
       <c r="C124" s="8" t="s">
-        <v>37</v>
+        <v>190</v>
       </c>
       <c r="D124" s="5">
-        <v>5</v>
+        <v>30</v>
       </c>
       <c r="E124" s="6" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="F124" s="4" t="s">
         <v>36</v>
@@ -3456,10 +3414,10 @@
       </c>
       <c r="B125" s="4"/>
       <c r="C125" s="8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D125" s="5">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="E125" s="6" t="s">
         <v>15</v>
@@ -3474,10 +3432,10 @@
       </c>
       <c r="B126" s="4"/>
       <c r="C126" s="8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D126" s="5">
-        <v>60</v>
+        <v>5</v>
       </c>
       <c r="E126" s="6" t="s">
         <v>15</v>
@@ -3492,13 +3450,13 @@
       </c>
       <c r="B127" s="4"/>
       <c r="C127" s="8" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D127" s="5">
         <v>10</v>
       </c>
       <c r="E127" s="6" t="s">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="F127" s="4" t="s">
         <v>36</v>
@@ -3510,13 +3468,13 @@
       </c>
       <c r="B128" s="4"/>
       <c r="C128" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D128" s="5">
-        <v>20</v>
+        <v>60</v>
       </c>
       <c r="E128" s="6" t="s">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="F128" s="4" t="s">
         <v>36</v>
@@ -3528,10 +3486,10 @@
       </c>
       <c r="B129" s="4"/>
       <c r="C129" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D129" s="5">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="E129" s="6" t="s">
         <v>7</v>
@@ -3546,7 +3504,7 @@
       </c>
       <c r="B130" s="4"/>
       <c r="C130" s="8" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D130" s="5">
         <v>20</v>
@@ -3564,10 +3522,10 @@
       </c>
       <c r="B131" s="4"/>
       <c r="C131" s="8" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D131" s="5">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="E131" s="6" t="s">
         <v>7</v>
@@ -3582,10 +3540,10 @@
       </c>
       <c r="B132" s="4"/>
       <c r="C132" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="D132" s="7">
-        <v>1000</v>
+        <v>44</v>
+      </c>
+      <c r="D132" s="5">
+        <v>20</v>
       </c>
       <c r="E132" s="6" t="s">
         <v>7</v>
@@ -3600,10 +3558,10 @@
       </c>
       <c r="B133" s="4"/>
       <c r="C133" s="8" t="s">
-        <v>201</v>
+        <v>45</v>
       </c>
       <c r="D133" s="5">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="E133" s="6" t="s">
         <v>7</v>
@@ -3620,8 +3578,8 @@
       <c r="C134" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="D134" s="5">
-        <v>10</v>
+      <c r="D134" s="7">
+        <v>1000</v>
       </c>
       <c r="E134" s="6" t="s">
         <v>7</v>
@@ -3639,7 +3597,7 @@
         <v>47</v>
       </c>
       <c r="D135" s="5">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="E135" s="6" t="s">
         <v>15</v>
@@ -3654,10 +3612,10 @@
       </c>
       <c r="B136" s="4"/>
       <c r="C136" s="8" t="s">
-        <v>49</v>
+        <v>191</v>
       </c>
       <c r="D136" s="5">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E136" s="6" t="s">
         <v>15</v>
@@ -3690,10 +3648,10 @@
       </c>
       <c r="B138" s="4"/>
       <c r="C138" s="8" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D138" s="5">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="E138" s="6" t="s">
         <v>15</v>
@@ -3708,10 +3666,10 @@
       </c>
       <c r="B139" s="4"/>
       <c r="C139" s="8" t="s">
-        <v>202</v>
+        <v>50</v>
       </c>
       <c r="D139" s="5">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E139" s="6" t="s">
         <v>15</v>
@@ -3744,7 +3702,7 @@
       </c>
       <c r="B141" s="4"/>
       <c r="C141" s="8" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D141" s="5">
         <v>6</v>
@@ -3765,7 +3723,7 @@
         <v>51</v>
       </c>
       <c r="D142" s="5">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="E142" s="6" t="s">
         <v>52</v>
@@ -3783,10 +3741,10 @@
         <v>53</v>
       </c>
       <c r="D143" s="5">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="E143" s="6" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="F143" s="4" t="s">
         <v>48</v>
@@ -3798,13 +3756,13 @@
       </c>
       <c r="B144" s="4"/>
       <c r="C144" s="8" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D144" s="5">
         <v>10</v>
       </c>
       <c r="E144" s="6" t="s">
-        <v>15</v>
+        <v>55</v>
       </c>
       <c r="F144" s="4" t="s">
         <v>48</v>
@@ -3819,10 +3777,10 @@
         <v>56</v>
       </c>
       <c r="D145" s="5">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E145" s="6" t="s">
-        <v>52</v>
+        <v>15</v>
       </c>
       <c r="F145" s="4" t="s">
         <v>48</v>
@@ -3834,7 +3792,7 @@
       </c>
       <c r="B146" s="4"/>
       <c r="C146" s="8" t="s">
-        <v>203</v>
+        <v>192</v>
       </c>
       <c r="D146" s="5">
         <v>2</v>
@@ -3852,7 +3810,7 @@
       </c>
       <c r="B147" s="4"/>
       <c r="C147" s="8" t="s">
-        <v>204</v>
+        <v>193</v>
       </c>
       <c r="D147" s="5">
         <v>6</v>
@@ -3870,10 +3828,10 @@
       </c>
       <c r="B148" s="4"/>
       <c r="C148" s="8" t="s">
-        <v>205</v>
-      </c>
-      <c r="D148" s="5">
-        <v>100</v>
+        <v>194</v>
+      </c>
+      <c r="D148" s="7">
+        <v>4000</v>
       </c>
       <c r="E148" s="6" t="s">
         <v>7</v>
@@ -3888,7 +3846,7 @@
       </c>
       <c r="B149" s="4"/>
       <c r="C149" s="8" t="s">
-        <v>206</v>
+        <v>195</v>
       </c>
       <c r="D149" s="5">
         <v>100</v>
@@ -3906,7 +3864,7 @@
       </c>
       <c r="B150" s="4"/>
       <c r="C150" s="8" t="s">
-        <v>207</v>
+        <v>196</v>
       </c>
       <c r="D150" s="5">
         <v>200</v>
@@ -3924,7 +3882,7 @@
       </c>
       <c r="B151" s="4"/>
       <c r="C151" s="8" t="s">
-        <v>208</v>
+        <v>197</v>
       </c>
       <c r="D151" s="5">
         <v>100</v>
@@ -3942,10 +3900,10 @@
       </c>
       <c r="B152" s="4"/>
       <c r="C152" s="8" t="s">
-        <v>209</v>
-      </c>
-      <c r="D152" s="7">
-        <v>4000</v>
+        <v>198</v>
+      </c>
+      <c r="D152" s="5">
+        <v>100</v>
       </c>
       <c r="E152" s="6" t="s">
         <v>7</v>
@@ -3960,13 +3918,13 @@
       </c>
       <c r="B153" s="4"/>
       <c r="C153" s="8" t="s">
-        <v>210</v>
+        <v>199</v>
       </c>
       <c r="D153" s="5">
-        <v>3</v>
+        <v>29</v>
       </c>
       <c r="E153" s="6" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="F153" s="4" t="s">
         <v>59</v>
@@ -3978,10 +3936,10 @@
       </c>
       <c r="B154" s="4"/>
       <c r="C154" s="8" t="s">
-        <v>211</v>
+        <v>200</v>
       </c>
       <c r="D154" s="5">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E154" s="6" t="s">
         <v>7</v>
@@ -3996,10 +3954,10 @@
       </c>
       <c r="B155" s="4"/>
       <c r="C155" s="8" t="s">
-        <v>212</v>
+        <v>201</v>
       </c>
       <c r="D155" s="5">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E155" s="6" t="s">
         <v>7</v>
@@ -4014,10 +3972,10 @@
       </c>
       <c r="B156" s="4"/>
       <c r="C156" s="8" t="s">
-        <v>213</v>
+        <v>202</v>
       </c>
       <c r="D156" s="5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E156" s="6" t="s">
         <v>7</v>
@@ -4032,10 +3990,10 @@
       </c>
       <c r="B157" s="4"/>
       <c r="C157" s="8" t="s">
-        <v>214</v>
+        <v>203</v>
       </c>
       <c r="D157" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E157" s="6" t="s">
         <v>7</v>
@@ -4050,10 +4008,10 @@
       </c>
       <c r="B158" s="4"/>
       <c r="C158" s="8" t="s">
-        <v>215</v>
+        <v>204</v>
       </c>
       <c r="D158" s="5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E158" s="6" t="s">
         <v>7</v>
@@ -4068,13 +4026,13 @@
       </c>
       <c r="B159" s="4"/>
       <c r="C159" s="8" t="s">
-        <v>216</v>
+        <v>205</v>
       </c>
       <c r="D159" s="5">
-        <v>29</v>
+        <v>3</v>
       </c>
       <c r="E159" s="6" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="F159" s="4" t="s">
         <v>59</v>
@@ -4104,7 +4062,7 @@
       </c>
       <c r="B161" s="4"/>
       <c r="C161" s="8" t="s">
-        <v>217</v>
+        <v>206</v>
       </c>
       <c r="D161" s="5">
         <v>800</v>
@@ -4122,10 +4080,10 @@
       </c>
       <c r="B162" s="4"/>
       <c r="C162" s="8" t="s">
-        <v>218</v>
+        <v>207</v>
       </c>
       <c r="D162" s="5">
-        <v>300</v>
+        <v>400</v>
       </c>
       <c r="E162" s="6" t="s">
         <v>7</v>
@@ -4140,7 +4098,7 @@
       </c>
       <c r="B163" s="4"/>
       <c r="C163" s="8" t="s">
-        <v>219</v>
+        <v>208</v>
       </c>
       <c r="D163" s="5">
         <v>300</v>
@@ -4158,10 +4116,10 @@
       </c>
       <c r="B164" s="4"/>
       <c r="C164" s="8" t="s">
-        <v>220</v>
+        <v>209</v>
       </c>
       <c r="D164" s="5">
-        <v>400</v>
+        <v>300</v>
       </c>
       <c r="E164" s="6" t="s">
         <v>7</v>
@@ -4176,7 +4134,7 @@
       </c>
       <c r="B165" s="4"/>
       <c r="C165" s="8" t="s">
-        <v>221</v>
+        <v>210</v>
       </c>
       <c r="D165" s="5">
         <v>800</v>
@@ -4197,10 +4155,10 @@
         <v>63</v>
       </c>
       <c r="D166" s="5">
-        <v>200</v>
+        <v>4</v>
       </c>
       <c r="E166" s="6" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="F166" s="4" t="s">
         <v>64</v>
@@ -4212,13 +4170,13 @@
       </c>
       <c r="B167" s="4"/>
       <c r="C167" s="8" t="s">
-        <v>222</v>
-      </c>
-      <c r="D167" s="5">
-        <v>3</v>
+        <v>211</v>
+      </c>
+      <c r="D167" s="7">
+        <v>2713.44</v>
       </c>
       <c r="E167" s="6" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="F167" s="4" t="s">
         <v>65</v>
@@ -4230,13 +4188,13 @@
       </c>
       <c r="B168" s="4"/>
       <c r="C168" s="8" t="s">
-        <v>223</v>
+        <v>212</v>
       </c>
       <c r="D168" s="5">
-        <v>48</v>
+        <v>35.28</v>
       </c>
       <c r="E168" s="6" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="F168" s="4" t="s">
         <v>65</v>
@@ -4248,13 +4206,13 @@
       </c>
       <c r="B169" s="4"/>
       <c r="C169" s="8" t="s">
-        <v>224</v>
+        <v>213</v>
       </c>
       <c r="D169" s="5">
-        <v>450</v>
+        <v>66</v>
       </c>
       <c r="E169" s="6" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="F169" s="4" t="s">
         <v>65</v>
@@ -4266,13 +4224,13 @@
       </c>
       <c r="B170" s="4"/>
       <c r="C170" s="8" t="s">
-        <v>225</v>
+        <v>214</v>
       </c>
       <c r="D170" s="5">
-        <v>48</v>
+        <v>5.82</v>
       </c>
       <c r="E170" s="6" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="F170" s="4" t="s">
         <v>65</v>
@@ -4284,13 +4242,13 @@
       </c>
       <c r="B171" s="4"/>
       <c r="C171" s="8" t="s">
-        <v>226</v>
+        <v>215</v>
       </c>
       <c r="D171" s="5">
-        <v>35</v>
+        <v>103.74</v>
       </c>
       <c r="E171" s="6" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="F171" s="4" t="s">
         <v>65</v>
@@ -4302,34 +4260,34 @@
       </c>
       <c r="B172" s="4"/>
       <c r="C172" s="8" t="s">
-        <v>227</v>
+        <v>216</v>
       </c>
       <c r="D172" s="5">
-        <v>25</v>
+        <v>20.22</v>
       </c>
       <c r="E172" s="6" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="F172" s="4" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="173" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="173" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A173" s="3">
         <v>172</v>
       </c>
       <c r="B173" s="4"/>
       <c r="C173" s="8" t="s">
-        <v>228</v>
+        <v>66</v>
       </c>
       <c r="D173" s="5">
-        <v>12</v>
+        <v>612</v>
       </c>
       <c r="E173" s="6" t="s">
-        <v>7</v>
+        <v>67</v>
       </c>
       <c r="F173" s="4" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
     </row>
     <row r="174" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -4338,16 +4296,16 @@
       </c>
       <c r="B174" s="4"/>
       <c r="C174" s="8" t="s">
-        <v>66</v>
+        <v>217</v>
       </c>
       <c r="D174" s="5">
-        <v>180</v>
+        <v>19.5</v>
       </c>
       <c r="E174" s="6" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="F174" s="4" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
     </row>
     <row r="175" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -4356,16 +4314,16 @@
       </c>
       <c r="B175" s="4"/>
       <c r="C175" s="8" t="s">
-        <v>67</v>
+        <v>218</v>
       </c>
       <c r="D175" s="5">
-        <v>450</v>
+        <v>1.8</v>
       </c>
       <c r="E175" s="6" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="F175" s="4" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
     </row>
     <row r="176" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -4374,16 +4332,16 @@
       </c>
       <c r="B176" s="4"/>
       <c r="C176" s="8" t="s">
-        <v>68</v>
+        <v>219</v>
       </c>
       <c r="D176" s="5">
-        <v>30</v>
+        <v>4</v>
       </c>
       <c r="E176" s="6" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="F176" s="4" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
     </row>
     <row r="177" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -4392,16 +4350,16 @@
       </c>
       <c r="B177" s="4"/>
       <c r="C177" s="8" t="s">
-        <v>69</v>
+        <v>220</v>
       </c>
       <c r="D177" s="5">
-        <v>30</v>
+        <v>4</v>
       </c>
       <c r="E177" s="6" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="F177" s="4" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
     </row>
     <row r="178" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -4410,16 +4368,16 @@
       </c>
       <c r="B178" s="4"/>
       <c r="C178" s="8" t="s">
+        <v>221</v>
+      </c>
+      <c r="D178" s="5">
+        <v>6</v>
+      </c>
+      <c r="E178" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="F178" s="4" t="s">
         <v>70</v>
-      </c>
-      <c r="D178" s="5">
-        <v>10</v>
-      </c>
-      <c r="E178" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="F178" s="4" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="179" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -4428,16 +4386,16 @@
       </c>
       <c r="B179" s="4"/>
       <c r="C179" s="8" t="s">
-        <v>71</v>
+        <v>222</v>
       </c>
       <c r="D179" s="5">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E179" s="6" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="F179" s="4" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
     </row>
     <row r="180" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -4446,16 +4404,16 @@
       </c>
       <c r="B180" s="4"/>
       <c r="C180" s="8" t="s">
-        <v>72</v>
+        <v>233</v>
       </c>
       <c r="D180" s="5">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="E180" s="6" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="F180" s="4" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
     </row>
     <row r="181" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -4464,16 +4422,16 @@
       </c>
       <c r="B181" s="4"/>
       <c r="C181" s="8" t="s">
-        <v>229</v>
+        <v>223</v>
       </c>
       <c r="D181" s="5">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="E181" s="6" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="F181" s="4" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
     </row>
     <row r="182" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -4482,16 +4440,16 @@
       </c>
       <c r="B182" s="4"/>
       <c r="C182" s="8" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="D182" s="5">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="E182" s="6" t="s">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="F182" s="4" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
     </row>
     <row r="183" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -4500,106 +4458,106 @@
       </c>
       <c r="B183" s="4"/>
       <c r="C183" s="8" t="s">
-        <v>230</v>
+        <v>73</v>
       </c>
       <c r="D183" s="5">
-        <v>32.799999999999997</v>
+        <v>3</v>
       </c>
       <c r="E183" s="6" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="F183" s="4" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="184" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="184" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A184" s="3">
         <v>183</v>
       </c>
       <c r="B184" s="4"/>
       <c r="C184" s="8" t="s">
+        <v>205</v>
+      </c>
+      <c r="D184" s="5">
+        <v>2</v>
+      </c>
+      <c r="E184" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="F184" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="D184" s="5">
-        <v>200</v>
-      </c>
-      <c r="E184" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="F184" s="4" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="185" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="185" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A185" s="3">
         <v>184</v>
       </c>
       <c r="B185" s="4"/>
       <c r="C185" s="8" t="s">
-        <v>231</v>
-      </c>
-      <c r="D185" s="7">
-        <v>1000</v>
+        <v>224</v>
+      </c>
+      <c r="D185" s="5">
+        <v>100</v>
       </c>
       <c r="E185" s="6" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="F185" s="4" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="186" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="186" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A186" s="3">
         <v>185</v>
       </c>
       <c r="B186" s="4"/>
       <c r="C186" s="8" t="s">
+        <v>225</v>
+      </c>
+      <c r="D186" s="5">
+        <v>100</v>
+      </c>
+      <c r="E186" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="F186" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="D186" s="7">
-        <v>3300</v>
-      </c>
-      <c r="E186" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="F186" s="4" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="187" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="187" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A187" s="3">
         <v>186</v>
       </c>
       <c r="B187" s="4"/>
       <c r="C187" s="8" t="s">
-        <v>77</v>
+        <v>226</v>
       </c>
       <c r="D187" s="5">
-        <v>1.1000000000000001</v>
+        <v>20</v>
       </c>
       <c r="E187" s="6" t="s">
-        <v>78</v>
+        <v>7</v>
       </c>
       <c r="F187" s="4" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="188" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="188" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A188" s="3">
         <v>187</v>
       </c>
       <c r="B188" s="4"/>
       <c r="C188" s="8" t="s">
-        <v>79</v>
+        <v>227</v>
       </c>
       <c r="D188" s="5">
-        <v>0.7</v>
+        <v>10</v>
       </c>
       <c r="E188" s="6" t="s">
-        <v>80</v>
+        <v>7</v>
       </c>
       <c r="F188" s="4" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="189" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -4608,70 +4566,70 @@
       </c>
       <c r="B189" s="4"/>
       <c r="C189" s="8" t="s">
-        <v>232</v>
+        <v>228</v>
       </c>
       <c r="D189" s="5">
-        <v>400</v>
+        <v>100</v>
       </c>
       <c r="E189" s="6" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="F189" s="4" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="190" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="190" spans="1:6" ht="35.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A190" s="3">
         <v>189</v>
       </c>
       <c r="B190" s="4"/>
       <c r="C190" s="8" t="s">
-        <v>81</v>
+        <v>229</v>
       </c>
       <c r="D190" s="5">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="E190" s="6" t="s">
-        <v>9</v>
+        <v>77</v>
       </c>
       <c r="F190" s="4" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="191" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="191" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A191" s="3">
         <v>190</v>
       </c>
       <c r="B191" s="4"/>
       <c r="C191" s="8" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="D191" s="5">
-        <v>1</v>
+        <v>36</v>
       </c>
       <c r="E191" s="6" t="s">
         <v>15</v>
       </c>
       <c r="F191" s="4" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="192" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="192" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A192" s="3">
         <v>191</v>
       </c>
       <c r="B192" s="4"/>
       <c r="C192" s="8" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="D192" s="5">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="E192" s="6" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="F192" s="4" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
     </row>
     <row r="193" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -4680,322 +4638,106 @@
       </c>
       <c r="B193" s="4"/>
       <c r="C193" s="8" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="D193" s="5">
-        <v>157.19999999999999</v>
+        <v>36</v>
       </c>
       <c r="E193" s="6" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="F193" s="4" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="194" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="194" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A194" s="3">
         <v>193</v>
       </c>
       <c r="B194" s="4"/>
       <c r="C194" s="8" t="s">
-        <v>234</v>
-      </c>
-      <c r="D194" s="7">
-        <v>2713.44</v>
+        <v>81</v>
+      </c>
+      <c r="D194" s="5">
+        <v>18</v>
       </c>
       <c r="E194" s="6" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="F194" s="4" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="195" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="195" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A195" s="3">
         <v>194</v>
       </c>
       <c r="B195" s="4"/>
       <c r="C195" s="8" t="s">
-        <v>235</v>
+        <v>82</v>
       </c>
       <c r="D195" s="5">
-        <v>35.28</v>
+        <v>36</v>
       </c>
       <c r="E195" s="6" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="F195" s="4" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="196" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="196" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A196" s="3">
         <v>195</v>
       </c>
       <c r="B196" s="4"/>
       <c r="C196" s="8" t="s">
-        <v>236</v>
+        <v>83</v>
       </c>
       <c r="D196" s="5">
-        <v>66</v>
+        <v>18</v>
       </c>
       <c r="E196" s="6" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="F196" s="4" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="197" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="197" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A197" s="3">
         <v>196</v>
       </c>
       <c r="B197" s="4"/>
       <c r="C197" s="8" t="s">
-        <v>237</v>
+        <v>231</v>
       </c>
       <c r="D197" s="5">
-        <v>5.82</v>
+        <v>36</v>
       </c>
       <c r="E197" s="6" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="F197" s="4" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="198" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="198" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A198" s="3">
         <v>197</v>
       </c>
       <c r="B198" s="4"/>
       <c r="C198" s="8" t="s">
-        <v>238</v>
+        <v>232</v>
       </c>
       <c r="D198" s="5">
-        <v>103.74</v>
+        <v>36</v>
       </c>
       <c r="E198" s="6" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="F198" s="4" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="199" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A199" s="3">
-        <v>198</v>
-      </c>
-      <c r="B199" s="4"/>
-      <c r="C199" s="8" t="s">
-        <v>239</v>
-      </c>
-      <c r="D199" s="5">
-        <v>20.22</v>
-      </c>
-      <c r="E199" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="F199" s="4" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="200" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A200" s="3">
-        <v>199</v>
-      </c>
-      <c r="B200" s="4"/>
-      <c r="C200" s="8" t="s">
-        <v>88</v>
-      </c>
-      <c r="D200" s="5">
-        <v>612</v>
-      </c>
-      <c r="E200" s="6" t="s">
-        <v>80</v>
-      </c>
-      <c r="F200" s="4" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="201" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A201" s="3">
-        <v>200</v>
-      </c>
-      <c r="B201" s="4"/>
-      <c r="C201" s="8" t="s">
-        <v>240</v>
-      </c>
-      <c r="D201" s="5">
-        <v>19.5</v>
-      </c>
-      <c r="E201" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="F201" s="4" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="202" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A202" s="3">
-        <v>201</v>
-      </c>
-      <c r="B202" s="4"/>
-      <c r="C202" s="8" t="s">
-        <v>241</v>
-      </c>
-      <c r="D202" s="5">
-        <v>1.8</v>
-      </c>
-      <c r="E202" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="F202" s="4" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="203" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A203" s="3">
-        <v>202</v>
-      </c>
-      <c r="B203" s="4"/>
-      <c r="C203" s="8" t="s">
-        <v>242</v>
-      </c>
-      <c r="D203" s="5">
-        <v>4</v>
-      </c>
-      <c r="E203" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="F203" s="4" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="204" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A204" s="3">
-        <v>203</v>
-      </c>
-      <c r="B204" s="4"/>
-      <c r="C204" s="8" t="s">
-        <v>243</v>
-      </c>
-      <c r="D204" s="5">
-        <v>4</v>
-      </c>
-      <c r="E204" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="F204" s="4" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="205" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A205" s="3">
-        <v>204</v>
-      </c>
-      <c r="B205" s="4"/>
-      <c r="C205" s="8" t="s">
-        <v>244</v>
-      </c>
-      <c r="D205" s="5">
-        <v>6</v>
-      </c>
-      <c r="E205" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="F205" s="4" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="206" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A206" s="3">
-        <v>205</v>
-      </c>
-      <c r="B206" s="4"/>
-      <c r="C206" s="8" t="s">
-        <v>245</v>
-      </c>
-      <c r="D206" s="5">
-        <v>2</v>
-      </c>
-      <c r="E206" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="F206" s="4" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="207" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A207" s="3">
-        <v>206</v>
-      </c>
-      <c r="B207" s="4"/>
-      <c r="C207" s="8" t="s">
-        <v>247</v>
-      </c>
-      <c r="D207" s="5">
-        <v>2</v>
-      </c>
-      <c r="E207" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="F207" s="4" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="208" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A208" s="3">
-        <v>207</v>
-      </c>
-      <c r="B208" s="4"/>
-      <c r="C208" s="8" t="s">
-        <v>246</v>
-      </c>
-      <c r="D208" s="5">
-        <v>4</v>
-      </c>
-      <c r="E208" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="F208" s="4" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="209" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A209" s="3">
-        <v>208</v>
-      </c>
-      <c r="B209" s="4"/>
-      <c r="C209" s="8" t="s">
-        <v>92</v>
-      </c>
-      <c r="D209" s="5">
-        <v>25</v>
-      </c>
-      <c r="E209" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="F209" s="4" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="210" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A210" s="3">
-        <v>209</v>
-      </c>
-      <c r="B210" s="4"/>
-      <c r="C210" s="8" t="s">
-        <v>94</v>
-      </c>
-      <c r="D210" s="5">
-        <v>30</v>
-      </c>
-      <c r="E210" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="F210" s="4" t="s">
-        <v>93</v>
+        <v>79</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
new About and Footer
</commit_message>
<xml_diff>
--- a/public/procurement.xlsx
+++ b/public/procurement.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lka\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19AD3BCB-6882-40CB-BE56-C90C1CB4DE3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{673FD8E4-332E-4635-8F56-8C8C65B1E925}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="597" uniqueCount="234">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="573" uniqueCount="224">
   <si>
     <t>№ п/п</t>
   </si>
@@ -96,108 +96,108 @@
     <t>Ремонт двери 1900х1000мм(уст.ка вент. решеток, установка цепи и фиксатора, покраска)</t>
   </si>
   <si>
+    <t>ЛГУП-7654</t>
+  </si>
+  <si>
+    <t>мм</t>
+  </si>
+  <si>
+    <t>Комплект кабельной проходки МКС</t>
+  </si>
+  <si>
+    <t>компл</t>
+  </si>
+  <si>
+    <t>г</t>
+  </si>
+  <si>
+    <t>Резьбовой крепежный элемент с наружной резьбой РКН-20 У2 IP54 ЗЭТА</t>
+  </si>
+  <si>
     <t>Лампа индикации ADDS D22 LED белая 220В AC/DC ЛK-22 IP55 25152DEK Dekraft</t>
   </si>
   <si>
-    <t>ЛГУП-7654</t>
-  </si>
-  <si>
-    <t>Резьбовой крепежный элемент с наружной резьбой РКН-20 У2 IP54 ЗЭТА</t>
+    <t>Извещатель пожарный тепловой взрывозащищенный 101-07е 1Ex db [ia Ga] IIC Т4 Gb Х IP66</t>
+  </si>
+  <si>
+    <t>Винт для обеспечения электрического контакта крышек ( М 5 х 8) арт.CM030508</t>
+  </si>
+  <si>
+    <t>Аварийное освещение Вега 60 с БАП 2Ex Тех 1ExmbIIC T6 Gb X, IP65</t>
+  </si>
+  <si>
+    <t>Пломба 1-6х10-АД-1М ГОСТ 18677-73</t>
   </si>
   <si>
     <t>Электроприв четвер.взры. ГЗ-ОФВ-300/28М 1х220 DN80PN63 L=452 УХЛ (исп. фл. J)</t>
   </si>
   <si>
-    <t>Аварийное освещение Вега 60 с БАП 2Ex Тех 1ExmbIIC T6 Gb X, IP65</t>
-  </si>
-  <si>
-    <t>Пломба 1-6х10-АД-1М ГОСТ 18677-73</t>
-  </si>
-  <si>
-    <t>г</t>
-  </si>
-  <si>
-    <t>Комплект кабельной проходки МКС</t>
-  </si>
-  <si>
-    <t>компл</t>
-  </si>
-  <si>
-    <t>мм</t>
-  </si>
-  <si>
-    <t>Извещатель пожарный тепловой взрывозащищенный 101-07е 1Ex db [ia Ga] IIC Т4 Gb Х IP66</t>
-  </si>
-  <si>
-    <t>Винт для обеспечения электрического контакта крышек ( М 5 х 8) арт.CM030508</t>
+    <t>Бита (вставка) Spline М 8  L=30мм</t>
+  </si>
+  <si>
+    <t>ЛГУП-7867</t>
+  </si>
+  <si>
+    <t>Ветошь /рул./</t>
+  </si>
+  <si>
+    <t>Пленка воздушно-пузырчатая 1500мм*100 пог.м 2 сл (рул)</t>
+  </si>
+  <si>
+    <t>Маркер белый Paint 4мм</t>
+  </si>
+  <si>
+    <t>Кисточка 2 см</t>
+  </si>
+  <si>
+    <t>Кисточка 5 см</t>
+  </si>
+  <si>
+    <t>Кисточка 10 см</t>
+  </si>
+  <si>
+    <t>Стрейч пленка 500мм*185м</t>
+  </si>
+  <si>
+    <t>Рулетка 3м (Force) (100)</t>
+  </si>
+  <si>
+    <t>Перчатки 4нит. 10кл. (черные) (пара)</t>
   </si>
   <si>
     <t>Рулетка  7,5м х 25мм обрезиненный корпус (3 фиксатора, зацеп с магнитом)</t>
   </si>
   <si>
-    <t>ЛГУП-7867</t>
-  </si>
-  <si>
-    <t>Бита (вставка) Spline М 8  L=30мм</t>
-  </si>
-  <si>
-    <t>Ветошь /рул./</t>
-  </si>
-  <si>
-    <t>Пленка воздушно-пузырчатая 1500мм*100 пог.м 2 сл (рул)</t>
-  </si>
-  <si>
-    <t>Маркер белый Paint 4мм</t>
-  </si>
-  <si>
-    <t>Кисточка 2 см</t>
-  </si>
-  <si>
-    <t>Кисточка 5 см</t>
-  </si>
-  <si>
-    <t>Кисточка 10 см</t>
-  </si>
-  <si>
-    <t>Стрейч пленка 500мм*185м</t>
-  </si>
-  <si>
-    <t>Рулетка 3м (Force) (100)</t>
-  </si>
-  <si>
-    <t>Перчатки 4нит. 10кл. (черные) (пара)</t>
+    <t>Паронит 3 мм</t>
+  </si>
+  <si>
+    <t>лист</t>
+  </si>
+  <si>
+    <t>НТУП-018192</t>
+  </si>
+  <si>
+    <t>Паронит 2мм</t>
+  </si>
+  <si>
+    <t>Ключи обмедненные</t>
+  </si>
+  <si>
+    <t>набор</t>
+  </si>
+  <si>
+    <t>Маркер по металлу белый</t>
+  </si>
+  <si>
+    <t>Маркер по металлу красный</t>
+  </si>
+  <si>
+    <t>Мел сварщика белый</t>
   </si>
   <si>
     <t>Маркер по металлу черный тонкий</t>
   </si>
   <si>
-    <t>НТУП-018192</t>
-  </si>
-  <si>
-    <t>Маркер по металлу белый</t>
-  </si>
-  <si>
-    <t>Маркер по металлу красный</t>
-  </si>
-  <si>
-    <t>Паронит 3 мм</t>
-  </si>
-  <si>
-    <t>лист</t>
-  </si>
-  <si>
-    <t>Паронит 2мм</t>
-  </si>
-  <si>
-    <t>Ключи обмедненные</t>
-  </si>
-  <si>
-    <t>набор</t>
-  </si>
-  <si>
-    <t>Мел сварщика белый</t>
-  </si>
-  <si>
     <t>ЛГУП-7998</t>
   </si>
   <si>
@@ -207,12 +207,6 @@
     <t>ЛГУП-8008</t>
   </si>
   <si>
-    <t>Штуцер Ш2.7038.001 (покрытие Хим.Фас)</t>
-  </si>
-  <si>
-    <t>ЛГУП-8012</t>
-  </si>
-  <si>
     <t>ЛГУП-8015</t>
   </si>
   <si>
@@ -240,43 +234,37 @@
     <t>ЛГУП-8046</t>
   </si>
   <si>
-    <t>Индустриальное масло  Gazpromneft  Industrial 40 ( И-40А ) 205л</t>
-  </si>
-  <si>
-    <t>ЛГУП-8058</t>
-  </si>
-  <si>
-    <t>Кран шаровый ДУ80 Ру 40 под приварку</t>
-  </si>
-  <si>
-    <t>НТУП-018299</t>
-  </si>
-  <si>
     <t>ЛГУП-8060</t>
   </si>
   <si>
-    <t>ЛГУП-8061</t>
-  </si>
-  <si>
-    <t>(не исп1) шт</t>
-  </si>
-  <si>
-    <t>Шайба 5Л ГОСТ 6402-70</t>
-  </si>
-  <si>
-    <t>ЛГУП-8062</t>
-  </si>
-  <si>
-    <t>Коробка соединительно-разветвительная взрывозащищенная КСРВ-2-2/0-К</t>
-  </si>
-  <si>
-    <t>Текстолит 4мм (90х60)</t>
-  </si>
-  <si>
-    <t>Саморез-шуруп острый (оцинк.) 2,2х4,5 ГОСТ 1144-80</t>
-  </si>
-  <si>
-    <t>Стойка для печатных плат (шестигр., латунь) М4, 27мм ГОСТ 20862-81</t>
+    <t>ЛГУП-8075</t>
+  </si>
+  <si>
+    <t>ЛГУП-8077</t>
+  </si>
+  <si>
+    <t>спец одежда  для специалистов ПНР (зимняя)</t>
+  </si>
+  <si>
+    <t>ЛГУП-8078</t>
+  </si>
+  <si>
+    <t>Патрубок (361)</t>
+  </si>
+  <si>
+    <t>ТЛУП-012027</t>
+  </si>
+  <si>
+    <t>Масло Лукойл 5w -40 4л</t>
+  </si>
+  <si>
+    <t>Тормозная жидкость</t>
+  </si>
+  <si>
+    <t>Масло  Лукойл -Авангард Ультра 5W40 CI-4/SL  п.синт /л/</t>
+  </si>
+  <si>
+    <t>Антифриз  felix</t>
   </si>
   <si>
     <t>Гофрокороб 395*155*155</t>
@@ -366,12 +354,12 @@
     <t>Круг D75 Ст.35 ГОСТ 1050-88</t>
   </si>
   <si>
+    <t>Круг D42 Ст.14Х17Н2 ГОСТ 5949-75</t>
+  </si>
+  <si>
     <t>Круг D75 Ст.20Х13 ГОСТ 5632-72</t>
   </si>
   <si>
-    <t>Круг D42 Ст.14Х17Н2 ГОСТ 5949-75</t>
-  </si>
-  <si>
     <t>Круг D20 Ст.20 ГОСТ 1050-88</t>
   </si>
   <si>
@@ -396,207 +384,207 @@
     <t>Газоанализатор взрывозащищенный СГОЭС (метан) 1Ex d IIC T4 Gb, IP67 Ур1. 10%, ур.2 50% НКПР</t>
   </si>
   <si>
+    <t>Коробка клеммная МТ Р407(-60+40) 2-8х20НК(А)-8х20НК(С)-2,5х31(П),1ЕхеLLCGbXT6, ip66, 220х120х90</t>
+  </si>
+  <si>
+    <t>Коробка клеммная МТ Р403(-60+40) 2-4х20НК(А)-4х20НК(С)-2,5х20(П),1ЕхеLLCGbXT6, ip66, 160х175х55</t>
+  </si>
+  <si>
+    <t>Коробка клеммная МТ Р402(-60+40)12-2х20НК(А)-2х20НК(С)-1,5х11(П), 1ЕхеLLCGbXT6, ip66, 110х75х55</t>
+  </si>
+  <si>
+    <t>Коробка клеммная МТ Р307(-60+40) 2-6х20НК(А)-1х20НК(В)-6х20НК(С)-4х26(П) 1ЕхеLLCGbXT6, ip66</t>
+  </si>
+  <si>
+    <t>Консоль с опорой ML 300мм (шт)</t>
+  </si>
+  <si>
+    <t>Компрессионный блок МКС КБ 120</t>
+  </si>
+  <si>
+    <t>Кабель-канал 10453 Legrand DPL 195х65 (2м)</t>
+  </si>
+  <si>
+    <t>Крышка Угол горизонтальный CPO 90 (50х50)</t>
+  </si>
+  <si>
+    <t>Трубка для фильтра 1/4" Гейзер</t>
+  </si>
+  <si>
+    <t>Лента самоклеящаяся уплотнительная ППЭ 5х15 МКС</t>
+  </si>
+  <si>
+    <t>Заглушка 10707 Legrand DPL 65х195</t>
+  </si>
+  <si>
+    <t>Заглушка  25х25 для трубы профильной ПВД черная</t>
+  </si>
+  <si>
+    <t>Диод КД209А ТТЗ.362.008 ТУ</t>
+  </si>
+  <si>
+    <t>Держатель проводника Rd8, DEHNGRIP NIRO h20 с отв.8мм М6</t>
+  </si>
+  <si>
+    <t>Припой с канифолью ПОС 61 d=1,0мм ГОСТ 21931-76 (Sn61; Pb39)</t>
+  </si>
+  <si>
+    <t>Уплотнительный модуль МКС 40/Ø 17-34 мм</t>
+  </si>
+  <si>
+    <t>Уплотнительный модуль МКС 20/О 5-14мм</t>
+  </si>
+  <si>
+    <t>Угол горизонтальный CPO 90 (50 х 50)</t>
+  </si>
+  <si>
+    <t>Наконечник НВИ 2-5 вилка 1,5-2,5мм SQ0503-0005 TDM</t>
+  </si>
+  <si>
+    <t>MV-клемма проводника Rd8</t>
+  </si>
+  <si>
+    <t>Плата питания ПСМ.11.00.00.01-02</t>
+  </si>
+  <si>
+    <t>Плата печатная ПСМ.11.00.01.01-02</t>
+  </si>
+  <si>
+    <t>Пластина для заземления PTCE арт. 37501</t>
+  </si>
+  <si>
+    <t>Пластина анкерная 120</t>
+  </si>
+  <si>
+    <t>Ответная рама РВО 4.1.1</t>
+  </si>
+  <si>
+    <t>Ответная рама РВО 2.1.1</t>
+  </si>
+  <si>
+    <t>Монтажная рама РВМ 4.1.1</t>
+  </si>
+  <si>
+    <t>Монтажная рама РВМ 2.1.1</t>
+  </si>
+  <si>
+    <t>Металлический лоток, неперфорированный (50х50х3000)</t>
+  </si>
+  <si>
+    <t>Металлический лоток, неперфорированный (100х50х3000)</t>
+  </si>
+  <si>
+    <t>Кабель ВВГнг(А)-LS-ХЛ 3x1,5 d7,2мм</t>
+  </si>
+  <si>
+    <t>Кабель ВВГнг(А)-LS- 3х2,50</t>
+  </si>
+  <si>
+    <t>Короб ПВХ 100х60</t>
+  </si>
+  <si>
+    <t>Короб ПВХ  40х25 мм</t>
+  </si>
+  <si>
+    <t>Кабель КПСЭнг(А)-FRLS 2*2*0,75</t>
+  </si>
+  <si>
+    <t>Кабель КПСЭнг(A)-FRLS 4х2х0,75</t>
+  </si>
+  <si>
+    <t>Кабель КВВГЭнг(А)-LS-ХЛ 7х1,0</t>
+  </si>
+  <si>
+    <t>Кабель КВВГЭнг(А)-LS-ХЛ 4х1,0</t>
+  </si>
+  <si>
+    <t>Кабель ВВГнг(А)-LS-ХЛ 4x1,5 d10,2мм</t>
+  </si>
+  <si>
+    <t>Трубка 3.31 ТВ-40 ГОСТ 19034-82</t>
+  </si>
+  <si>
+    <t>Провод НВМ 0,35 IV 500 ГОСТ 17515-72</t>
+  </si>
+  <si>
+    <t>Кабель ВВГнг(А)-FRLS 3x1,5 d7,2мм</t>
+  </si>
+  <si>
+    <t>Кабель ВВГнг(А)-LS-ХЛ 3x2,5 d8мм</t>
+  </si>
+  <si>
+    <t>Провод желто-зеленый ПуГВнг(А)-LS 1x6,0</t>
+  </si>
+  <si>
+    <t>Короб ПВХ 40х40 мм</t>
+  </si>
+  <si>
+    <t>Провод желто-зеленый ПуГВнг(А)-LS 1x25</t>
+  </si>
+  <si>
+    <t>Провод Rd8</t>
+  </si>
+  <si>
+    <t>Металлорукав в ПВХ изоляции РЗ-ЦП-15</t>
+  </si>
+  <si>
+    <t>Аварийное освещение Вега 60 2Ex Тех  IP65</t>
+  </si>
+  <si>
     <t>Аварийное освещение DL-0128A 28 Вт IP65</t>
   </si>
   <si>
-    <t>Аварийное освещение Вега 60 2Ex Тех  IP65</t>
-  </si>
-  <si>
-    <t>Крышка Угол горизонтальный CPO 90 (50х50)</t>
-  </si>
-  <si>
-    <t>Металлический лоток, неперфорированный (100х50х3000)</t>
-  </si>
-  <si>
-    <t>Металлический лоток, неперфорированный (50х50х3000)</t>
-  </si>
-  <si>
-    <t>Монтажная рама РВМ 2.1.1</t>
-  </si>
-  <si>
-    <t>Монтажная рама РВМ 4.1.1</t>
-  </si>
-  <si>
-    <t>Ответная рама РВО 2.1.1</t>
-  </si>
-  <si>
-    <t>Ответная рама РВО 4.1.1</t>
-  </si>
-  <si>
-    <t>Пластина анкерная 120</t>
-  </si>
-  <si>
-    <t>Пластина для заземления PTCE арт. 37501</t>
-  </si>
-  <si>
-    <t>Плата печатная ПСМ.11.00.01.01-02</t>
-  </si>
-  <si>
-    <t>Плата питания ПСМ.11.00.00.01-02</t>
-  </si>
-  <si>
-    <t>Угол горизонтальный CPO 90 (50 х 50)</t>
-  </si>
-  <si>
-    <t>Уплотнительный модуль МКС 20/О 5-14мм</t>
-  </si>
-  <si>
-    <t>Уплотнительный модуль МКС 40/Ø 17-34 мм</t>
-  </si>
-  <si>
-    <t>Наконечник НВИ 2-5 вилка 1,5-2,5мм SQ0503-0005 TDM</t>
-  </si>
-  <si>
-    <t>Припой с канифолью ПОС 61 d=1,0мм ГОСТ 21931-76 (Sn61; Pb39)</t>
-  </si>
-  <si>
-    <t>Держатель проводника Rd8, DEHNGRIP NIRO h20 с отв.8мм М6</t>
-  </si>
-  <si>
-    <t>Диод КД209А ТТЗ.362.008 ТУ</t>
-  </si>
-  <si>
-    <t>Заглушка  25х25 для трубы профильной ПВД черная</t>
-  </si>
-  <si>
-    <t>Заглушка 10707 Legrand DPL 65х195</t>
-  </si>
-  <si>
-    <t>Лента самоклеящаяся уплотнительная ППЭ 5х15 МКС</t>
-  </si>
-  <si>
-    <t>Трубка для фильтра 1/4" Гейзер</t>
-  </si>
-  <si>
-    <t>MV-клемма проводника Rd8</t>
-  </si>
-  <si>
-    <t>Кабель-канал 10453 Legrand DPL 195х65 (2м)</t>
-  </si>
-  <si>
-    <t>Компрессионный блок МКС КБ 120</t>
-  </si>
-  <si>
-    <t>Консоль с опорой ML 300мм (шт)</t>
-  </si>
-  <si>
-    <t>Коробка клеммная МТ Р307(-60+40) 2-6х20НК(А)-1х20НК(В)-6х20НК(С)-4х26(П) 1ЕхеLLCGbXT6, ip66</t>
-  </si>
-  <si>
-    <t>Коробка клеммная МТ Р402(-60+40)12-2х20НК(А)-2х20НК(С)-1,5х11(П), 1ЕхеLLCGbXT6, ip66, 110х75х55</t>
-  </si>
-  <si>
-    <t>Коробка клеммная МТ Р403(-60+40) 2-4х20НК(А)-4х20НК(С)-2,5х20(П),1ЕхеLLCGbXT6, ip66, 160х175х55</t>
-  </si>
-  <si>
-    <t>Коробка клеммная МТ Р407(-60+40) 2-8х20НК(А)-8х20НК(С)-2,5х31(П),1ЕхеLLCGbXT6, ip66, 220х120х90</t>
-  </si>
-  <si>
-    <t>Короб ПВХ 40х40 мм</t>
-  </si>
-  <si>
-    <t>Провод желто-зеленый ПуГВнг(А)-LS 1x6,0</t>
-  </si>
-  <si>
-    <t>Кабель ВВГнг(А)-LS-ХЛ 3x2,5 d8мм</t>
-  </si>
-  <si>
-    <t>Кабель ВВГнг(А)-LS-ХЛ 3x1,5 d7,2мм</t>
-  </si>
-  <si>
-    <t>Кабель ВВГнг(А)-LS- 3х2,50</t>
-  </si>
-  <si>
-    <t>Короб ПВХ 100х60</t>
-  </si>
-  <si>
-    <t>Короб ПВХ  40х25 мм</t>
-  </si>
-  <si>
-    <t>Кабель КПСЭнг(А)-FRLS 2*2*0,75</t>
-  </si>
-  <si>
-    <t>Кабель КПСЭнг(A)-FRLS 4х2х0,75</t>
-  </si>
-  <si>
-    <t>Кабель КВВГЭнг(А)-LS-ХЛ 7х1,0</t>
-  </si>
-  <si>
-    <t>Кабель КВВГЭнг(А)-LS-ХЛ 4х1,0</t>
-  </si>
-  <si>
-    <t>Кабель ВВГнг(А)-LS-ХЛ 4x1,5 d10,2мм</t>
-  </si>
-  <si>
-    <t>Трубка 3.31 ТВ-40 ГОСТ 19034-82</t>
-  </si>
-  <si>
-    <t>Провод НВМ 0,35 IV 500 ГОСТ 17515-72</t>
-  </si>
-  <si>
-    <t>Кабель ВВГнг(А)-FRLS 3x1,5 d7,2мм</t>
-  </si>
-  <si>
-    <t>Провод желто-зеленый ПуГВнг(А)-LS 1x25</t>
-  </si>
-  <si>
-    <t>Провод Rd8</t>
-  </si>
-  <si>
-    <t>Металлорукав в ПВХ изоляции РЗ-ЦП-15</t>
+    <t>Держатель для полосы заземления К-188 У2 (цинк)</t>
+  </si>
+  <si>
+    <t>Геркон КЭМ-2</t>
+  </si>
+  <si>
+    <t>Коробка клеммная МТ Р407(-60+40) 2-8х20НК(А)-8х20НК(С)-4х26(П),1ЕхеLLCGbXT6, ip66, 220х120х90</t>
+  </si>
+  <si>
+    <t>Коробка распаячная КМ41242 IP55</t>
+  </si>
+  <si>
+    <t>Крепление для труб ПВХ с защелкой, 16 мм</t>
+  </si>
+  <si>
+    <t>Крышка (100х15х3000)</t>
+  </si>
+  <si>
+    <t>Крышка (50х15х3000)</t>
+  </si>
+  <si>
+    <t>Крышка на Угол вертикальный внешний CD 90 (50 х 50)</t>
+  </si>
+  <si>
+    <t>Крышка Угол горизонтальный CPO 90 (100х50)</t>
+  </si>
+  <si>
+    <t>Профиль PSM (3000) арт. 34181</t>
+  </si>
+  <si>
+    <t>Резьбовой крепежный элемент с внутренней резьбой Ркв-15</t>
+  </si>
+  <si>
+    <t>Резьбовой крепежный элемент с наружной резьбой РКН-15 (ММРн-15)</t>
+  </si>
+  <si>
+    <t>Скоба металлическая СМО 16-17 49152 КВТ</t>
+  </si>
+  <si>
+    <t>Считыватель бесконтактный для proxi-карт, Proxy-3МA IP20</t>
+  </si>
+  <si>
+    <t>Считыватель бесконтактный для proxi-карт, RD 26-REH-КМ АЯКС Ex mb IIC T5 Gb X , IP67</t>
+  </si>
+  <si>
+    <t>Угол горизонтальный CPO 90 (100 х 50)</t>
   </si>
   <si>
     <t>Выключатель двухклавишный IP55</t>
   </si>
   <si>
-    <t>Геркон КЭМ-2</t>
-  </si>
-  <si>
-    <t>Держатель для полосы заземления К-188 У2 (цинк)</t>
-  </si>
-  <si>
-    <t>Угол горизонтальный CPO 90 (100 х 50)</t>
-  </si>
-  <si>
-    <t>Считыватель бесконтактный для proxi-карт, RD 26-REH-КМ АЯКС Ex mb IIC T5 Gb X , IP67</t>
-  </si>
-  <si>
-    <t>Считыватель бесконтактный для proxi-карт, Proxy-3МA IP20</t>
-  </si>
-  <si>
-    <t>Скоба металлическая СМО 16-17 49152 КВТ</t>
-  </si>
-  <si>
-    <t>Резьбовой крепежный элемент с наружной резьбой РКН-15 (ММРн-15)</t>
-  </si>
-  <si>
-    <t>Резьбовой крепежный элемент с внутренней резьбой Ркв-15</t>
-  </si>
-  <si>
-    <t>Профиль PSM (3000) арт. 34181</t>
-  </si>
-  <si>
-    <t>Коробка клеммная МТ Р407(-60+40) 2-8х20НК(А)-8х20НК(С)-4х26(П),1ЕхеLLCGbXT6, ip66, 220х120х90</t>
-  </si>
-  <si>
-    <t>Коробка распаячная КМ41242 IP55</t>
-  </si>
-  <si>
-    <t>Крышка Угол горизонтальный CPO 90 (100х50)</t>
-  </si>
-  <si>
-    <t>Крышка на Угол вертикальный внешний CD 90 (50 х 50)</t>
-  </si>
-  <si>
-    <t>Крышка (50х15х3000)</t>
-  </si>
-  <si>
-    <t>Крышка (100х15х3000)</t>
-  </si>
-  <si>
-    <t>Крепление для труб ПВХ с защелкой, 16 мм</t>
-  </si>
-  <si>
     <t>Очки защитные для токарей.О15.</t>
   </si>
   <si>
@@ -609,57 +597,57 @@
     <t>Пост аварийной сигнализации загазованности в/защ.ПАСВ1-П-75-1Ж1К-В1 (=24В, -60..+40С) 1ExsIICT6</t>
   </si>
   <si>
+    <t>Пружина НТ.3.02.00.00.002-01</t>
+  </si>
+  <si>
+    <t>Пружина №467 НТ.200.000.029.0</t>
+  </si>
+  <si>
+    <t>Пружина крышки НТ.200.004.003.0</t>
+  </si>
+  <si>
+    <t>Пружина №442 НТ.110.000.007.0</t>
+  </si>
+  <si>
     <t>Магнит МС3 ЦО 14,5/4 ТУ 3498-005-12591667-2014</t>
   </si>
   <si>
-    <t>Пружина №442 НТ.110.000.007.0</t>
-  </si>
-  <si>
-    <t>Пружина крышки НТ.200.004.003.0</t>
-  </si>
-  <si>
-    <t>Пружина №467 НТ.200.000.029.0</t>
-  </si>
-  <si>
-    <t>Пружина НТ.3.02.00.00.002-01</t>
-  </si>
-  <si>
     <t>Грунт-эмаль Дюропокс ДТМ 80 (внутрянка)</t>
   </si>
   <si>
+    <t>Легкосбрасываемое окнная конструкция 1200х1100 мм / ПВХ-профили морозост. исп, RAL 9003 белый</t>
+  </si>
+  <si>
+    <t>Задвижка ЗКС 31лс77нж Ду 15 Ру 40 МПа (соединение муфтовое Rc 1/2)</t>
+  </si>
+  <si>
+    <t>Задвижка клиновая литая ЗКЛ 50-40 УХЛ1 30С15нж, класс герм.А (ряд 2, исп.фл.3)</t>
+  </si>
+  <si>
+    <t>Задвижка клиновая литая ЗКЛ 80-40 УХЛ1 30лс15нж, класс герм.А (ряд 2, исп.фл.3)</t>
+  </si>
+  <si>
+    <t>Клапан обратный поворотный КОП 80-40 УХЛ1 19лс53нж (исп. фл. 3)</t>
+  </si>
+  <si>
     <t>Дверь левс доводчиком2000х1000мм(ВхШ) полотно RAL 9003(белый)/коробка(RAL 9003)(белый)с цепью</t>
   </si>
   <si>
-    <t>Клапан обратный поворотный КОП 80-40 УХЛ1 19лс53нж (исп. фл. 3)</t>
-  </si>
-  <si>
-    <t>Задвижка клиновая литая ЗКЛ 80-40 УХЛ1 30лс15нж, класс герм.А (ряд 2, исп.фл.3)</t>
-  </si>
-  <si>
-    <t>Легкосбрасываемое окнная конструкция 1200х1100 мм / ПВХ-профили морозост. исп, RAL 9003 белый</t>
-  </si>
-  <si>
-    <t>Задвижка клиновая литая ЗКЛ 50-40 УХЛ1 30С15нж, класс герм.А (ряд 2, исп.фл.3)</t>
-  </si>
-  <si>
-    <t>Задвижка ЗКС 31лс77нж Ду 15 Ру 40 МПа (соединение муфтовое Rc 1/2)</t>
+    <t>Гайка М16-6Н.8.20.019 ГОСТ 15523-70</t>
+  </si>
+  <si>
+    <t>Гайка М14х1,5 ГОСТ 15522-70</t>
+  </si>
+  <si>
+    <t>Гайка М10.5 019 ГОСТ 5927-70</t>
+  </si>
+  <si>
+    <t>Гайка М10-6Н ГОСТ 5927-70 (размер под ключ S=17)</t>
   </si>
   <si>
     <t>Болт М8-6gх25.58.019 ГОСТ 7798-70</t>
   </si>
   <si>
-    <t>Гайка М10-6Н ГОСТ 5927-70 (размер под ключ S=17)</t>
-  </si>
-  <si>
-    <t>Гайка М10.5 019 ГОСТ 5927-70</t>
-  </si>
-  <si>
-    <t>Гайка М14х1,5 ГОСТ 15522-70</t>
-  </si>
-  <si>
-    <t>Гайка М16-6Н.8.20.019 ГОСТ 15523-70</t>
-  </si>
-  <si>
     <t>Лист чечевица В-К-ПУ-3,0 Ст.09Г2С ГОСТ 8568-77</t>
   </si>
   <si>
@@ -684,46 +672,28 @@
     <t>Лист Б-ПР-1,0 ГОСТ 19904-74/ 4-III-Ст3кп ГОСТ 16523-89</t>
   </si>
   <si>
+    <t>Кольцо уплотнительное НТ 202.003.004.0</t>
+  </si>
+  <si>
+    <t>Кольцо А18х1,2 ГОСТ 13942-86</t>
+  </si>
+  <si>
+    <t>Кольцо 070-076-36 ГОСТ 9833-73</t>
+  </si>
+  <si>
+    <t>Кольцо 038-042-25 ГОСТ 9833-70</t>
+  </si>
+  <si>
     <t>Кольцо 035-041-36-2-4 ГОСТ 9833-73</t>
   </si>
   <si>
-    <t>Кольцо 038-042-25 ГОСТ 9833-70</t>
-  </si>
-  <si>
-    <t>Кольцо 070-076-36 ГОСТ 9833-73</t>
-  </si>
-  <si>
-    <t>Кольцо А18х1,2 ГОСТ 13942-86</t>
-  </si>
-  <si>
-    <t>Кольцо уплотнительное НТ 202.003.004.0</t>
-  </si>
-  <si>
-    <t>Пластина WNMG 080408-GP GM3225 GESAC</t>
-  </si>
-  <si>
-    <t>Пластина CCMT09T308-GP GM3225 GESAC</t>
-  </si>
-  <si>
-    <t>Пластина SPGT060204-DG AT9030</t>
-  </si>
-  <si>
-    <t>Фреза концевая твердосплавная GE-D10.0-25L-4F-10D-75L</t>
-  </si>
-  <si>
-    <t>Пластина R390-11 T3 08M-PM 1130 SANDVIK (кратно12 для корпуса ПСМ, кратно 2 -для верх.корп.КМР)</t>
-  </si>
-  <si>
-    <t>Фреза концевая твердосплавная D5*HRC55*L100*25*4F</t>
-  </si>
-  <si>
-    <t>Винт М4х6 ГОСТ 17473-80</t>
-  </si>
-  <si>
-    <t>Болт М5х40 оцинк. ГОСТ 7805-70</t>
-  </si>
-  <si>
-    <t>Шайба 5.01.019 ГОСТ 11371-78</t>
+    <t>Державка SNR0010K11</t>
+  </si>
+  <si>
+    <t>Пластина 11IR2.00ISO BT2225</t>
+  </si>
+  <si>
+    <t>Кабель ВВГ 3*2,5</t>
   </si>
   <si>
     <t>Кольцо А75х1,7 ГОСТ 13943-86_</t>
@@ -1163,12 +1133,12 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr autoPageBreaks="0" fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F198"/>
+  <dimension ref="A1:F190"/>
   <sheetFormatPr defaultColWidth="10.5" defaultRowHeight="11.45" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="5.1640625" style="1" customWidth="1"/>
     <col min="2" max="2" width="46.6640625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="74.83203125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="75" style="1" customWidth="1"/>
     <col min="4" max="4" width="14.1640625" style="1" customWidth="1"/>
     <col min="5" max="5" width="13" style="1" customWidth="1"/>
     <col min="6" max="6" width="14.5" style="1" customWidth="1"/>
@@ -1218,7 +1188,7 @@
       </c>
       <c r="B3" s="4"/>
       <c r="C3" s="8" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="D3" s="5">
         <v>15</v>
@@ -1236,7 +1206,7 @@
       </c>
       <c r="B4" s="4"/>
       <c r="C4" s="8" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="D4" s="5">
         <v>9</v>
@@ -1254,7 +1224,7 @@
       </c>
       <c r="B5" s="4"/>
       <c r="C5" s="8" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="D5" s="5">
         <v>21</v>
@@ -1272,7 +1242,7 @@
       </c>
       <c r="B6" s="4"/>
       <c r="C6" s="8" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="D6" s="5">
         <v>60</v>
@@ -1290,7 +1260,7 @@
       </c>
       <c r="B7" s="4"/>
       <c r="C7" s="8" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="D7" s="5">
         <v>6</v>
@@ -1308,7 +1278,7 @@
       </c>
       <c r="B8" s="4"/>
       <c r="C8" s="8" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="D8" s="5">
         <v>0.75</v>
@@ -1326,7 +1296,7 @@
       </c>
       <c r="B9" s="4"/>
       <c r="C9" s="8" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="D9" s="5">
         <v>5.4</v>
@@ -1344,7 +1314,7 @@
       </c>
       <c r="B10" s="4"/>
       <c r="C10" s="8" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="D10" s="5">
         <v>0.33</v>
@@ -1362,7 +1332,7 @@
       </c>
       <c r="B11" s="4"/>
       <c r="C11" s="8" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="D11" s="5">
         <v>0.15</v>
@@ -1380,7 +1350,7 @@
       </c>
       <c r="B12" s="4"/>
       <c r="C12" s="8" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="D12" s="5">
         <v>6.6</v>
@@ -1398,7 +1368,7 @@
       </c>
       <c r="B13" s="4"/>
       <c r="C13" s="8" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="D13" s="5">
         <v>3.6</v>
@@ -1416,7 +1386,7 @@
       </c>
       <c r="B14" s="4"/>
       <c r="C14" s="8" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="D14" s="5">
         <v>36.9</v>
@@ -1434,7 +1404,7 @@
       </c>
       <c r="B15" s="4"/>
       <c r="C15" s="8" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D15" s="5">
         <v>0.3</v>
@@ -1452,7 +1422,7 @@
       </c>
       <c r="B16" s="4"/>
       <c r="C16" s="8" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="D16" s="5">
         <v>52.05</v>
@@ -1470,7 +1440,7 @@
       </c>
       <c r="B17" s="4"/>
       <c r="C17" s="8" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="D17" s="5">
         <v>90</v>
@@ -1488,7 +1458,7 @@
       </c>
       <c r="B18" s="4"/>
       <c r="C18" s="8" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="D18" s="5">
         <v>47.4</v>
@@ -1506,7 +1476,7 @@
       </c>
       <c r="B19" s="4"/>
       <c r="C19" s="8" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="D19" s="5">
         <v>15.9</v>
@@ -1524,7 +1494,7 @@
       </c>
       <c r="B20" s="4"/>
       <c r="C20" s="8" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="D20" s="5">
         <v>472.8</v>
@@ -1542,7 +1512,7 @@
       </c>
       <c r="B21" s="4"/>
       <c r="C21" s="8" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="D21" s="5">
         <v>112.8</v>
@@ -1578,7 +1548,7 @@
       </c>
       <c r="B23" s="4"/>
       <c r="C23" s="8" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="D23" s="5">
         <v>20.7</v>
@@ -1596,7 +1566,7 @@
       </c>
       <c r="B24" s="4"/>
       <c r="C24" s="8" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="D24" s="5">
         <v>22.5</v>
@@ -1614,7 +1584,7 @@
       </c>
       <c r="B25" s="4"/>
       <c r="C25" s="8" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="D25" s="5">
         <v>13.65</v>
@@ -1632,7 +1602,7 @@
       </c>
       <c r="B26" s="4"/>
       <c r="C26" s="8" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="D26" s="5">
         <v>21.9</v>
@@ -1650,7 +1620,7 @@
       </c>
       <c r="B27" s="4"/>
       <c r="C27" s="8" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="D27" s="5">
         <v>6.6</v>
@@ -1668,7 +1638,7 @@
       </c>
       <c r="B28" s="4"/>
       <c r="C28" s="8" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="D28" s="5">
         <v>0.09</v>
@@ -1686,7 +1656,7 @@
       </c>
       <c r="B29" s="4"/>
       <c r="C29" s="8" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="D29" s="5">
         <v>55.8</v>
@@ -1704,7 +1674,7 @@
       </c>
       <c r="B30" s="4"/>
       <c r="C30" s="8" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="D30" s="5">
         <v>20.399999999999999</v>
@@ -1722,7 +1692,7 @@
       </c>
       <c r="B31" s="4"/>
       <c r="C31" s="8" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D31" s="5">
         <v>40.5</v>
@@ -1740,7 +1710,7 @@
       </c>
       <c r="B32" s="4"/>
       <c r="C32" s="8" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="D32" s="5">
         <v>33.15</v>
@@ -1758,10 +1728,10 @@
       </c>
       <c r="B33" s="4"/>
       <c r="C33" s="8" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="D33" s="5">
-        <v>20.7</v>
+        <v>38.700000000000003</v>
       </c>
       <c r="E33" s="6" t="s">
         <v>11</v>
@@ -1776,10 +1746,10 @@
       </c>
       <c r="B34" s="4"/>
       <c r="C34" s="8" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="D34" s="5">
-        <v>38.700000000000003</v>
+        <v>20.7</v>
       </c>
       <c r="E34" s="6" t="s">
         <v>11</v>
@@ -1794,7 +1764,7 @@
       </c>
       <c r="B35" s="4"/>
       <c r="C35" s="8" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="D35" s="5">
         <v>1.05</v>
@@ -1848,7 +1818,7 @@
       </c>
       <c r="B38" s="4"/>
       <c r="C38" s="8" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="D38" s="5">
         <v>200</v>
@@ -1866,7 +1836,7 @@
       </c>
       <c r="B39" s="4"/>
       <c r="C39" s="8" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="D39" s="5">
         <v>200</v>
@@ -1884,7 +1854,7 @@
       </c>
       <c r="B40" s="4"/>
       <c r="C40" s="8" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="D40" s="5">
         <v>200</v>
@@ -1902,7 +1872,7 @@
       </c>
       <c r="B41" s="4"/>
       <c r="C41" s="8" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="D41" s="5">
         <v>200</v>
@@ -1920,7 +1890,7 @@
       </c>
       <c r="B42" s="4"/>
       <c r="C42" s="8" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="D42" s="5">
         <v>200</v>
@@ -1938,7 +1908,7 @@
       </c>
       <c r="B43" s="4"/>
       <c r="C43" s="8" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="D43" s="5">
         <v>200</v>
@@ -1956,7 +1926,7 @@
       </c>
       <c r="B44" s="4"/>
       <c r="C44" s="8" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="D44" s="5">
         <v>1</v>
@@ -2004,76 +1974,76 @@
         <v>21</v>
       </c>
     </row>
-    <row r="47" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="3">
         <v>46</v>
       </c>
       <c r="B47" s="4"/>
       <c r="C47" s="8" t="s">
-        <v>23</v>
+        <v>119</v>
       </c>
       <c r="D47" s="5">
-        <v>153</v>
+        <v>10</v>
       </c>
       <c r="E47" s="6" t="s">
         <v>7</v>
       </c>
       <c r="F47" s="4" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="48" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="3">
         <v>47</v>
       </c>
       <c r="B48" s="4"/>
       <c r="C48" s="8" t="s">
-        <v>25</v>
+        <v>120</v>
       </c>
       <c r="D48" s="5">
-        <v>42</v>
+        <v>10</v>
       </c>
       <c r="E48" s="6" t="s">
         <v>7</v>
       </c>
       <c r="F48" s="4" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="49" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="3">
         <v>48</v>
       </c>
       <c r="B49" s="4"/>
       <c r="C49" s="8" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="D49" s="5">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E49" s="6" t="s">
         <v>7</v>
       </c>
       <c r="F49" s="4" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="50" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="3">
         <v>49</v>
       </c>
       <c r="B50" s="4"/>
       <c r="C50" s="8" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="D50" s="5">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="E50" s="6" t="s">
         <v>7</v>
       </c>
       <c r="F50" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="51" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2082,16 +2052,16 @@
       </c>
       <c r="B51" s="4"/>
       <c r="C51" s="8" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="D51" s="5">
-        <v>64</v>
+        <v>112</v>
       </c>
       <c r="E51" s="6" t="s">
         <v>7</v>
       </c>
       <c r="F51" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="52" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2100,16 +2070,16 @@
       </c>
       <c r="B52" s="4"/>
       <c r="C52" s="8" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="D52" s="5">
-        <v>57</v>
+        <v>16</v>
       </c>
       <c r="E52" s="6" t="s">
         <v>7</v>
       </c>
       <c r="F52" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="53" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2118,16 +2088,16 @@
       </c>
       <c r="B53" s="4"/>
       <c r="C53" s="8" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="D53" s="5">
-        <v>144</v>
+        <v>40</v>
       </c>
       <c r="E53" s="6" t="s">
         <v>7</v>
       </c>
       <c r="F53" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="54" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2136,16 +2106,16 @@
       </c>
       <c r="B54" s="4"/>
       <c r="C54" s="8" t="s">
-        <v>26</v>
+        <v>126</v>
       </c>
       <c r="D54" s="5">
-        <v>6</v>
+        <v>64</v>
       </c>
       <c r="E54" s="6" t="s">
         <v>7</v>
       </c>
       <c r="F54" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="55" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2154,16 +2124,16 @@
       </c>
       <c r="B55" s="4"/>
       <c r="C55" s="8" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D55" s="5">
-        <v>8</v>
+        <v>48</v>
       </c>
       <c r="E55" s="6" t="s">
-        <v>7</v>
+        <v>24</v>
       </c>
       <c r="F55" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="56" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2172,16 +2142,16 @@
       </c>
       <c r="B56" s="4"/>
       <c r="C56" s="8" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D56" s="5">
-        <v>8</v>
+        <v>16.8</v>
       </c>
       <c r="E56" s="6" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F56" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="57" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2190,16 +2160,16 @@
       </c>
       <c r="B57" s="4"/>
       <c r="C57" s="8" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D57" s="5">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E57" s="6" t="s">
         <v>7</v>
       </c>
       <c r="F57" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="58" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2208,16 +2178,16 @@
       </c>
       <c r="B58" s="4"/>
       <c r="C58" s="8" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D58" s="5">
-        <v>8</v>
+        <v>76</v>
       </c>
       <c r="E58" s="6" t="s">
         <v>7</v>
       </c>
       <c r="F58" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="59" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2226,16 +2196,16 @@
       </c>
       <c r="B59" s="4"/>
       <c r="C59" s="8" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D59" s="5">
-        <v>56</v>
+        <v>192</v>
       </c>
       <c r="E59" s="6" t="s">
         <v>7</v>
       </c>
       <c r="F59" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="60" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2244,16 +2214,16 @@
       </c>
       <c r="B60" s="4"/>
       <c r="C60" s="8" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D60" s="5">
-        <v>200</v>
+        <v>560</v>
       </c>
       <c r="E60" s="6" t="s">
         <v>7</v>
       </c>
       <c r="F60" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="61" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2262,16 +2232,16 @@
       </c>
       <c r="B61" s="4"/>
       <c r="C61" s="8" t="s">
-        <v>134</v>
+        <v>25</v>
       </c>
       <c r="D61" s="5">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="E61" s="6" t="s">
-        <v>7</v>
+        <v>26</v>
       </c>
       <c r="F61" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="62" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2280,16 +2250,16 @@
       </c>
       <c r="B62" s="4"/>
       <c r="C62" s="8" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="D62" s="5">
-        <v>8</v>
+        <v>88</v>
       </c>
       <c r="E62" s="6" t="s">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="F62" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="63" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2298,16 +2268,16 @@
       </c>
       <c r="B63" s="4"/>
       <c r="C63" s="8" t="s">
-        <v>27</v>
+        <v>134</v>
       </c>
       <c r="D63" s="5">
-        <v>6</v>
+        <v>48</v>
       </c>
       <c r="E63" s="6" t="s">
         <v>7</v>
       </c>
       <c r="F63" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="64" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2316,16 +2286,16 @@
       </c>
       <c r="B64" s="4"/>
       <c r="C64" s="8" t="s">
-        <v>28</v>
+        <v>135</v>
       </c>
       <c r="D64" s="5">
-        <v>16</v>
+        <v>240</v>
       </c>
       <c r="E64" s="6" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="F64" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="65" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2343,7 +2313,7 @@
         <v>7</v>
       </c>
       <c r="F65" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="66" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2355,13 +2325,13 @@
         <v>137</v>
       </c>
       <c r="D66" s="5">
-        <v>240</v>
+        <v>40</v>
       </c>
       <c r="E66" s="6" t="s">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="F66" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="67" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2373,13 +2343,13 @@
         <v>138</v>
       </c>
       <c r="D67" s="5">
-        <v>48</v>
+        <v>32</v>
       </c>
       <c r="E67" s="6" t="s">
         <v>7</v>
       </c>
       <c r="F67" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="68" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2388,16 +2358,16 @@
       </c>
       <c r="B68" s="4"/>
       <c r="C68" s="8" t="s">
-        <v>139</v>
+        <v>28</v>
       </c>
       <c r="D68" s="5">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E68" s="6" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="F68" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="69" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2406,19 +2376,19 @@
       </c>
       <c r="B69" s="4"/>
       <c r="C69" s="8" t="s">
-        <v>140</v>
+        <v>29</v>
       </c>
       <c r="D69" s="5">
-        <v>88</v>
+        <v>153</v>
       </c>
       <c r="E69" s="6" t="s">
-        <v>29</v>
+        <v>7</v>
       </c>
       <c r="F69" s="4" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="70" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A70" s="3">
         <v>69</v>
       </c>
@@ -2427,13 +2397,13 @@
         <v>30</v>
       </c>
       <c r="D70" s="5">
-        <v>3</v>
+        <v>24</v>
       </c>
       <c r="E70" s="6" t="s">
-        <v>31</v>
+        <v>7</v>
       </c>
       <c r="F70" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="71" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2442,16 +2412,16 @@
       </c>
       <c r="B71" s="4"/>
       <c r="C71" s="8" t="s">
-        <v>141</v>
+        <v>31</v>
       </c>
       <c r="D71" s="5">
-        <v>560</v>
+        <v>160</v>
       </c>
       <c r="E71" s="6" t="s">
         <v>7</v>
       </c>
       <c r="F71" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="72" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2460,16 +2430,16 @@
       </c>
       <c r="B72" s="4"/>
       <c r="C72" s="8" t="s">
-        <v>142</v>
+        <v>32</v>
       </c>
       <c r="D72" s="5">
-        <v>192</v>
+        <v>6</v>
       </c>
       <c r="E72" s="6" t="s">
         <v>7</v>
       </c>
       <c r="F72" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="73" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2478,16 +2448,16 @@
       </c>
       <c r="B73" s="4"/>
       <c r="C73" s="8" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="D73" s="5">
-        <v>76</v>
+        <v>8</v>
       </c>
       <c r="E73" s="6" t="s">
         <v>7</v>
       </c>
       <c r="F73" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="74" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2496,16 +2466,16 @@
       </c>
       <c r="B74" s="4"/>
       <c r="C74" s="8" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="D74" s="5">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E74" s="6" t="s">
         <v>7</v>
       </c>
       <c r="F74" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="75" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2514,16 +2484,16 @@
       </c>
       <c r="B75" s="4"/>
       <c r="C75" s="8" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="D75" s="5">
-        <v>16.8</v>
+        <v>200</v>
       </c>
       <c r="E75" s="6" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="F75" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="76" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2532,16 +2502,16 @@
       </c>
       <c r="B76" s="4"/>
       <c r="C76" s="8" t="s">
-        <v>146</v>
+        <v>33</v>
       </c>
       <c r="D76" s="5">
-        <v>48</v>
+        <v>16</v>
       </c>
       <c r="E76" s="6" t="s">
-        <v>32</v>
+        <v>15</v>
       </c>
       <c r="F76" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="77" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2550,16 +2520,16 @@
       </c>
       <c r="B77" s="4"/>
       <c r="C77" s="8" t="s">
-        <v>147</v>
+        <v>34</v>
       </c>
       <c r="D77" s="5">
-        <v>32</v>
+        <v>6</v>
       </c>
       <c r="E77" s="6" t="s">
         <v>7</v>
       </c>
       <c r="F77" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="78" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2568,16 +2538,16 @@
       </c>
       <c r="B78" s="4"/>
       <c r="C78" s="8" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="D78" s="5">
-        <v>40</v>
+        <v>56</v>
       </c>
       <c r="E78" s="6" t="s">
         <v>7</v>
       </c>
       <c r="F78" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="79" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2586,16 +2556,16 @@
       </c>
       <c r="B79" s="4"/>
       <c r="C79" s="8" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="D79" s="5">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="E79" s="6" t="s">
         <v>7</v>
       </c>
       <c r="F79" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="80" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2604,88 +2574,88 @@
       </c>
       <c r="B80" s="4"/>
       <c r="C80" s="8" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="D80" s="5">
-        <v>112</v>
+        <v>8</v>
       </c>
       <c r="E80" s="6" t="s">
         <v>7</v>
       </c>
       <c r="F80" s="4" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="81" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A81" s="3">
         <v>80</v>
       </c>
       <c r="B81" s="4"/>
       <c r="C81" s="8" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="D81" s="5">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="E81" s="6" t="s">
         <v>7</v>
       </c>
       <c r="F81" s="4" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="82" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A82" s="3">
         <v>81</v>
       </c>
       <c r="B82" s="4"/>
       <c r="C82" s="8" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="D82" s="5">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E82" s="6" t="s">
         <v>7</v>
       </c>
       <c r="F82" s="4" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="83" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A83" s="3">
         <v>82</v>
       </c>
       <c r="B83" s="4"/>
       <c r="C83" s="8" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="D83" s="5">
-        <v>10</v>
+        <v>144</v>
       </c>
       <c r="E83" s="6" t="s">
         <v>7</v>
       </c>
       <c r="F83" s="4" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="84" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A84" s="3">
         <v>83</v>
       </c>
       <c r="B84" s="4"/>
       <c r="C84" s="8" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
       <c r="D84" s="5">
-        <v>10</v>
+        <v>57</v>
       </c>
       <c r="E84" s="6" t="s">
         <v>7</v>
       </c>
       <c r="F84" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="85" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2694,16 +2664,16 @@
       </c>
       <c r="B85" s="4"/>
       <c r="C85" s="8" t="s">
-        <v>155</v>
-      </c>
-      <c r="D85" s="5">
-        <v>40</v>
+        <v>149</v>
+      </c>
+      <c r="D85" s="7">
+        <v>1199</v>
       </c>
       <c r="E85" s="6" t="s">
         <v>10</v>
       </c>
       <c r="F85" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="86" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2712,16 +2682,16 @@
       </c>
       <c r="B86" s="4"/>
       <c r="C86" s="8" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="D86" s="5">
-        <v>320</v>
+        <v>56</v>
       </c>
       <c r="E86" s="6" t="s">
         <v>10</v>
       </c>
       <c r="F86" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="87" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2730,16 +2700,16 @@
       </c>
       <c r="B87" s="4"/>
       <c r="C87" s="8" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
       <c r="D87" s="5">
-        <v>100.8</v>
+        <v>10</v>
       </c>
       <c r="E87" s="6" t="s">
         <v>10</v>
       </c>
       <c r="F87" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="88" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2748,16 +2718,16 @@
       </c>
       <c r="B88" s="4"/>
       <c r="C88" s="8" t="s">
-        <v>158</v>
-      </c>
-      <c r="D88" s="7">
-        <v>1199</v>
+        <v>152</v>
+      </c>
+      <c r="D88" s="5">
+        <v>30</v>
       </c>
       <c r="E88" s="6" t="s">
         <v>10</v>
       </c>
       <c r="F88" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="89" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2766,16 +2736,16 @@
       </c>
       <c r="B89" s="4"/>
       <c r="C89" s="8" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
       <c r="D89" s="5">
-        <v>56</v>
+        <v>861.2</v>
       </c>
       <c r="E89" s="6" t="s">
         <v>10</v>
       </c>
       <c r="F89" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="90" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2784,16 +2754,16 @@
       </c>
       <c r="B90" s="4"/>
       <c r="C90" s="8" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="D90" s="5">
-        <v>10</v>
+        <v>98</v>
       </c>
       <c r="E90" s="6" t="s">
         <v>10</v>
       </c>
       <c r="F90" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="91" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2802,16 +2772,16 @@
       </c>
       <c r="B91" s="4"/>
       <c r="C91" s="8" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="D91" s="5">
-        <v>30</v>
+        <v>288</v>
       </c>
       <c r="E91" s="6" t="s">
         <v>10</v>
       </c>
       <c r="F91" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="92" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2820,16 +2790,16 @@
       </c>
       <c r="B92" s="4"/>
       <c r="C92" s="8" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
       <c r="D92" s="5">
-        <v>861.2</v>
+        <v>989</v>
       </c>
       <c r="E92" s="6" t="s">
         <v>10</v>
       </c>
       <c r="F92" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="93" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2838,16 +2808,16 @@
       </c>
       <c r="B93" s="4"/>
       <c r="C93" s="8" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
       <c r="D93" s="5">
-        <v>98</v>
+        <v>396.5</v>
       </c>
       <c r="E93" s="6" t="s">
         <v>10</v>
       </c>
       <c r="F93" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="94" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2856,16 +2826,16 @@
       </c>
       <c r="B94" s="4"/>
       <c r="C94" s="8" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
       <c r="D94" s="5">
-        <v>288</v>
+        <v>0.6</v>
       </c>
       <c r="E94" s="6" t="s">
         <v>10</v>
       </c>
       <c r="F94" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="95" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2874,16 +2844,16 @@
       </c>
       <c r="B95" s="4"/>
       <c r="C95" s="8" t="s">
-        <v>165</v>
+        <v>159</v>
       </c>
       <c r="D95" s="5">
-        <v>989</v>
+        <v>16</v>
       </c>
       <c r="E95" s="6" t="s">
         <v>10</v>
       </c>
       <c r="F95" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="96" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2892,16 +2862,16 @@
       </c>
       <c r="B96" s="4"/>
       <c r="C96" s="8" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="D96" s="5">
-        <v>396.5</v>
+        <v>274.8</v>
       </c>
       <c r="E96" s="6" t="s">
         <v>10</v>
       </c>
       <c r="F96" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="97" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2910,16 +2880,16 @@
       </c>
       <c r="B97" s="4"/>
       <c r="C97" s="8" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="D97" s="5">
-        <v>0.6</v>
+        <v>100.8</v>
       </c>
       <c r="E97" s="6" t="s">
         <v>10</v>
       </c>
       <c r="F97" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="98" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2928,16 +2898,16 @@
       </c>
       <c r="B98" s="4"/>
       <c r="C98" s="8" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
       <c r="D98" s="5">
-        <v>16</v>
+        <v>320</v>
       </c>
       <c r="E98" s="6" t="s">
         <v>10</v>
       </c>
       <c r="F98" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="99" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2946,16 +2916,16 @@
       </c>
       <c r="B99" s="4"/>
       <c r="C99" s="8" t="s">
-        <v>169</v>
+        <v>163</v>
       </c>
       <c r="D99" s="5">
-        <v>274.8</v>
+        <v>40</v>
       </c>
       <c r="E99" s="6" t="s">
         <v>10</v>
       </c>
       <c r="F99" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="100" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2964,7 +2934,7 @@
       </c>
       <c r="B100" s="4"/>
       <c r="C100" s="8" t="s">
-        <v>170</v>
+        <v>164</v>
       </c>
       <c r="D100" s="5">
         <v>48</v>
@@ -2973,7 +2943,7 @@
         <v>10</v>
       </c>
       <c r="F100" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="101" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2982,7 +2952,7 @@
       </c>
       <c r="B101" s="4"/>
       <c r="C101" s="8" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="D101" s="5">
         <v>259</v>
@@ -2991,7 +2961,7 @@
         <v>10</v>
       </c>
       <c r="F101" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="102" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3000,7 +2970,7 @@
       </c>
       <c r="B102" s="4"/>
       <c r="C102" s="8" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="D102" s="7">
         <v>1040</v>
@@ -3009,7 +2979,7 @@
         <v>10</v>
       </c>
       <c r="F102" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="103" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3018,7 +2988,7 @@
       </c>
       <c r="B103" s="4"/>
       <c r="C103" s="8" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="D103" s="5">
         <v>602.20000000000005</v>
@@ -3027,25 +2997,25 @@
         <v>10</v>
       </c>
       <c r="F103" s="4" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="104" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A104" s="3">
         <v>103</v>
       </c>
       <c r="B104" s="4"/>
       <c r="C104" s="8" t="s">
-        <v>33</v>
+        <v>167</v>
       </c>
       <c r="D104" s="5">
-        <v>24</v>
+        <v>5</v>
       </c>
       <c r="E104" s="6" t="s">
         <v>7</v>
       </c>
       <c r="F104" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="105" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3054,7 +3024,7 @@
       </c>
       <c r="B105" s="4"/>
       <c r="C105" s="8" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="D105" s="5">
         <v>8</v>
@@ -3063,7 +3033,7 @@
         <v>7</v>
       </c>
       <c r="F105" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="106" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3072,16 +3042,16 @@
       </c>
       <c r="B106" s="4"/>
       <c r="C106" s="8" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
       <c r="D106" s="5">
-        <v>112</v>
+        <v>400</v>
       </c>
       <c r="E106" s="6" t="s">
         <v>7</v>
       </c>
       <c r="F106" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="107" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3090,34 +3060,34 @@
       </c>
       <c r="B107" s="4"/>
       <c r="C107" s="8" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="D107" s="5">
-        <v>400</v>
+        <v>112</v>
       </c>
       <c r="E107" s="6" t="s">
         <v>7</v>
       </c>
       <c r="F107" s="4" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="108" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A108" s="3">
         <v>107</v>
       </c>
       <c r="B108" s="4"/>
       <c r="C108" s="8" t="s">
-        <v>34</v>
+        <v>171</v>
       </c>
       <c r="D108" s="5">
-        <v>160</v>
+        <v>5</v>
       </c>
       <c r="E108" s="6" t="s">
         <v>7</v>
       </c>
       <c r="F108" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="109" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3126,34 +3096,34 @@
       </c>
       <c r="B109" s="4"/>
       <c r="C109" s="8" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="D109" s="5">
-        <v>32</v>
+        <v>8</v>
       </c>
       <c r="E109" s="6" t="s">
         <v>7</v>
       </c>
       <c r="F109" s="4" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="110" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A110" s="3">
         <v>109</v>
       </c>
       <c r="B110" s="4"/>
       <c r="C110" s="8" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D110" s="5">
-        <v>8</v>
+        <v>75</v>
       </c>
       <c r="E110" s="6" t="s">
         <v>7</v>
       </c>
       <c r="F110" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="111" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3162,16 +3132,16 @@
       </c>
       <c r="B111" s="4"/>
       <c r="C111" s="8" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D111" s="5">
-        <v>8</v>
+        <v>57</v>
       </c>
       <c r="E111" s="6" t="s">
         <v>7</v>
       </c>
       <c r="F111" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="112" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3180,16 +3150,16 @@
       </c>
       <c r="B112" s="4"/>
       <c r="C112" s="8" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="D112" s="5">
-        <v>900</v>
+        <v>144</v>
       </c>
       <c r="E112" s="6" t="s">
         <v>7</v>
       </c>
       <c r="F112" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="113" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3198,16 +3168,16 @@
       </c>
       <c r="B113" s="4"/>
       <c r="C113" s="8" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="D113" s="5">
-        <v>422</v>
+        <v>32</v>
       </c>
       <c r="E113" s="6" t="s">
         <v>7</v>
       </c>
       <c r="F113" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="114" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3216,16 +3186,16 @@
       </c>
       <c r="B114" s="4"/>
       <c r="C114" s="8" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="D114" s="5">
-        <v>298</v>
+        <v>32</v>
       </c>
       <c r="E114" s="6" t="s">
         <v>7</v>
       </c>
       <c r="F114" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="115" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3234,7 +3204,7 @@
       </c>
       <c r="B115" s="4"/>
       <c r="C115" s="8" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="D115" s="5">
         <v>40</v>
@@ -3243,25 +3213,25 @@
         <v>7</v>
       </c>
       <c r="F115" s="4" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="116" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A116" s="3">
         <v>115</v>
       </c>
       <c r="B116" s="4"/>
       <c r="C116" s="8" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="D116" s="5">
-        <v>5</v>
+        <v>298</v>
       </c>
       <c r="E116" s="6" t="s">
         <v>7</v>
       </c>
       <c r="F116" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="117" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3270,16 +3240,16 @@
       </c>
       <c r="B117" s="4"/>
       <c r="C117" s="8" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="D117" s="5">
-        <v>8</v>
+        <v>422</v>
       </c>
       <c r="E117" s="6" t="s">
         <v>7</v>
       </c>
       <c r="F117" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="118" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3288,16 +3258,16 @@
       </c>
       <c r="B118" s="4"/>
       <c r="C118" s="8" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="D118" s="5">
-        <v>32</v>
+        <v>900</v>
       </c>
       <c r="E118" s="6" t="s">
         <v>7</v>
       </c>
       <c r="F118" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="119" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3306,34 +3276,34 @@
       </c>
       <c r="B119" s="4"/>
       <c r="C119" s="8" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="D119" s="5">
-        <v>32</v>
+        <v>8</v>
       </c>
       <c r="E119" s="6" t="s">
         <v>7</v>
       </c>
       <c r="F119" s="4" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="120" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A120" s="3">
         <v>119</v>
       </c>
       <c r="B120" s="4"/>
       <c r="C120" s="8" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="D120" s="5">
-        <v>144</v>
+        <v>8</v>
       </c>
       <c r="E120" s="6" t="s">
         <v>7</v>
       </c>
       <c r="F120" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="121" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3342,16 +3312,16 @@
       </c>
       <c r="B121" s="4"/>
       <c r="C121" s="8" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="D121" s="5">
-        <v>57</v>
+        <v>32</v>
       </c>
       <c r="E121" s="6" t="s">
         <v>7</v>
       </c>
       <c r="F121" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="122" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3360,16 +3330,16 @@
       </c>
       <c r="B122" s="4"/>
       <c r="C122" s="8" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="D122" s="5">
-        <v>75</v>
+        <v>8</v>
       </c>
       <c r="E122" s="6" t="s">
         <v>7</v>
       </c>
       <c r="F122" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="123" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3381,10 +3351,10 @@
         <v>35</v>
       </c>
       <c r="D123" s="5">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="E123" s="6" t="s">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="F123" s="4" t="s">
         <v>36</v>
@@ -3396,13 +3366,13 @@
       </c>
       <c r="B124" s="4"/>
       <c r="C124" s="8" t="s">
-        <v>190</v>
+        <v>37</v>
       </c>
       <c r="D124" s="5">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="E124" s="6" t="s">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="F124" s="4" t="s">
         <v>36</v>
@@ -3414,10 +3384,10 @@
       </c>
       <c r="B125" s="4"/>
       <c r="C125" s="8" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D125" s="5">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="E125" s="6" t="s">
         <v>15</v>
@@ -3432,10 +3402,10 @@
       </c>
       <c r="B126" s="4"/>
       <c r="C126" s="8" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D126" s="5">
-        <v>5</v>
+        <v>60</v>
       </c>
       <c r="E126" s="6" t="s">
         <v>15</v>
@@ -3450,13 +3420,13 @@
       </c>
       <c r="B127" s="4"/>
       <c r="C127" s="8" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D127" s="5">
         <v>10</v>
       </c>
       <c r="E127" s="6" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="F127" s="4" t="s">
         <v>36</v>
@@ -3468,13 +3438,13 @@
       </c>
       <c r="B128" s="4"/>
       <c r="C128" s="8" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D128" s="5">
-        <v>60</v>
+        <v>20</v>
       </c>
       <c r="E128" s="6" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="F128" s="4" t="s">
         <v>36</v>
@@ -3486,10 +3456,10 @@
       </c>
       <c r="B129" s="4"/>
       <c r="C129" s="8" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D129" s="5">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="E129" s="6" t="s">
         <v>7</v>
@@ -3504,7 +3474,7 @@
       </c>
       <c r="B130" s="4"/>
       <c r="C130" s="8" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D130" s="5">
         <v>20</v>
@@ -3522,10 +3492,10 @@
       </c>
       <c r="B131" s="4"/>
       <c r="C131" s="8" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D131" s="5">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="E131" s="6" t="s">
         <v>7</v>
@@ -3540,10 +3510,10 @@
       </c>
       <c r="B132" s="4"/>
       <c r="C132" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="D132" s="5">
-        <v>20</v>
+        <v>45</v>
+      </c>
+      <c r="D132" s="7">
+        <v>1000</v>
       </c>
       <c r="E132" s="6" t="s">
         <v>7</v>
@@ -3558,10 +3528,10 @@
       </c>
       <c r="B133" s="4"/>
       <c r="C133" s="8" t="s">
-        <v>45</v>
+        <v>186</v>
       </c>
       <c r="D133" s="5">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="E133" s="6" t="s">
         <v>7</v>
@@ -3578,8 +3548,8 @@
       <c r="C134" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="D134" s="7">
-        <v>1000</v>
+      <c r="D134" s="5">
+        <v>10</v>
       </c>
       <c r="E134" s="6" t="s">
         <v>7</v>
@@ -3597,13 +3567,13 @@
         <v>47</v>
       </c>
       <c r="D135" s="5">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="E135" s="6" t="s">
-        <v>15</v>
+        <v>48</v>
       </c>
       <c r="F135" s="4" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="136" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3612,16 +3582,16 @@
       </c>
       <c r="B136" s="4"/>
       <c r="C136" s="8" t="s">
-        <v>191</v>
+        <v>50</v>
       </c>
       <c r="D136" s="5">
-        <v>5</v>
+        <v>30</v>
       </c>
       <c r="E136" s="6" t="s">
-        <v>15</v>
+        <v>48</v>
       </c>
       <c r="F136" s="4" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="137" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3630,16 +3600,16 @@
       </c>
       <c r="B137" s="4"/>
       <c r="C137" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="D137" s="5">
+        <v>10</v>
+      </c>
+      <c r="E137" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="F137" s="4" t="s">
         <v>49</v>
-      </c>
-      <c r="D137" s="5">
-        <v>20</v>
-      </c>
-      <c r="E137" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="F137" s="4" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="138" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3648,16 +3618,16 @@
       </c>
       <c r="B138" s="4"/>
       <c r="C138" s="8" t="s">
-        <v>49</v>
+        <v>37</v>
       </c>
       <c r="D138" s="5">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E138" s="6" t="s">
         <v>15</v>
       </c>
       <c r="F138" s="4" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="139" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3666,7 +3636,7 @@
       </c>
       <c r="B139" s="4"/>
       <c r="C139" s="8" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="D139" s="5">
         <v>10</v>
@@ -3675,7 +3645,7 @@
         <v>15</v>
       </c>
       <c r="F139" s="4" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="140" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3684,7 +3654,7 @@
       </c>
       <c r="B140" s="4"/>
       <c r="C140" s="8" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="D140" s="5">
         <v>10</v>
@@ -3693,7 +3663,7 @@
         <v>15</v>
       </c>
       <c r="F140" s="4" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="141" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3702,16 +3672,16 @@
       </c>
       <c r="B141" s="4"/>
       <c r="C141" s="8" t="s">
-        <v>38</v>
+        <v>53</v>
       </c>
       <c r="D141" s="5">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E141" s="6" t="s">
         <v>15</v>
       </c>
       <c r="F141" s="4" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="142" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3720,16 +3690,16 @@
       </c>
       <c r="B142" s="4"/>
       <c r="C142" s="8" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D142" s="5">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="E142" s="6" t="s">
-        <v>52</v>
+        <v>15</v>
       </c>
       <c r="F142" s="4" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="143" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3738,16 +3708,16 @@
       </c>
       <c r="B143" s="4"/>
       <c r="C143" s="8" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D143" s="5">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="E143" s="6" t="s">
-        <v>52</v>
+        <v>15</v>
       </c>
       <c r="F143" s="4" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="144" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3756,16 +3726,16 @@
       </c>
       <c r="B144" s="4"/>
       <c r="C144" s="8" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="D144" s="5">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="E144" s="6" t="s">
-        <v>55</v>
+        <v>15</v>
       </c>
       <c r="F144" s="4" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="145" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3774,16 +3744,16 @@
       </c>
       <c r="B145" s="4"/>
       <c r="C145" s="8" t="s">
-        <v>56</v>
+        <v>187</v>
       </c>
       <c r="D145" s="5">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E145" s="6" t="s">
         <v>15</v>
       </c>
       <c r="F145" s="4" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="146" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3792,7 +3762,7 @@
       </c>
       <c r="B146" s="4"/>
       <c r="C146" s="8" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="D146" s="5">
         <v>2</v>
@@ -3801,7 +3771,7 @@
         <v>7</v>
       </c>
       <c r="F146" s="4" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="147" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3810,7 +3780,7 @@
       </c>
       <c r="B147" s="4"/>
       <c r="C147" s="8" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="D147" s="5">
         <v>6</v>
@@ -3828,10 +3798,10 @@
       </c>
       <c r="B148" s="4"/>
       <c r="C148" s="8" t="s">
-        <v>194</v>
-      </c>
-      <c r="D148" s="7">
-        <v>4000</v>
+        <v>190</v>
+      </c>
+      <c r="D148" s="5">
+        <v>100</v>
       </c>
       <c r="E148" s="6" t="s">
         <v>7</v>
@@ -3846,7 +3816,7 @@
       </c>
       <c r="B149" s="4"/>
       <c r="C149" s="8" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="D149" s="5">
         <v>100</v>
@@ -3864,7 +3834,7 @@
       </c>
       <c r="B150" s="4"/>
       <c r="C150" s="8" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="D150" s="5">
         <v>200</v>
@@ -3882,7 +3852,7 @@
       </c>
       <c r="B151" s="4"/>
       <c r="C151" s="8" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="D151" s="5">
         <v>100</v>
@@ -3900,10 +3870,10 @@
       </c>
       <c r="B152" s="4"/>
       <c r="C152" s="8" t="s">
-        <v>198</v>
-      </c>
-      <c r="D152" s="5">
-        <v>100</v>
+        <v>194</v>
+      </c>
+      <c r="D152" s="7">
+        <v>4000</v>
       </c>
       <c r="E152" s="6" t="s">
         <v>7</v>
@@ -3918,7 +3888,7 @@
       </c>
       <c r="B153" s="4"/>
       <c r="C153" s="8" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="D153" s="5">
         <v>29</v>
@@ -3936,10 +3906,10 @@
       </c>
       <c r="B154" s="4"/>
       <c r="C154" s="8" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="D154" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E154" s="6" t="s">
         <v>7</v>
@@ -3954,10 +3924,10 @@
       </c>
       <c r="B155" s="4"/>
       <c r="C155" s="8" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="D155" s="5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E155" s="6" t="s">
         <v>7</v>
@@ -3972,7 +3942,7 @@
       </c>
       <c r="B156" s="4"/>
       <c r="C156" s="8" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="D156" s="5">
         <v>3</v>
@@ -3990,10 +3960,10 @@
       </c>
       <c r="B157" s="4"/>
       <c r="C157" s="8" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="D157" s="5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E157" s="6" t="s">
         <v>7</v>
@@ -4008,10 +3978,10 @@
       </c>
       <c r="B158" s="4"/>
       <c r="C158" s="8" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="D158" s="5">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E158" s="6" t="s">
         <v>7</v>
@@ -4026,10 +3996,10 @@
       </c>
       <c r="B159" s="4"/>
       <c r="C159" s="8" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="D159" s="5">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E159" s="6" t="s">
         <v>7</v>
@@ -4038,22 +4008,22 @@
         <v>59</v>
       </c>
     </row>
-    <row r="160" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="160" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A160" s="3">
         <v>159</v>
       </c>
       <c r="B160" s="4"/>
       <c r="C160" s="8" t="s">
+        <v>202</v>
+      </c>
+      <c r="D160" s="5">
+        <v>800</v>
+      </c>
+      <c r="E160" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="F160" s="4" t="s">
         <v>60</v>
-      </c>
-      <c r="D160" s="5">
-        <v>1</v>
-      </c>
-      <c r="E160" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="F160" s="4" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="161" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -4062,16 +4032,16 @@
       </c>
       <c r="B161" s="4"/>
       <c r="C161" s="8" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="D161" s="5">
-        <v>800</v>
+        <v>300</v>
       </c>
       <c r="E161" s="6" t="s">
         <v>7</v>
       </c>
       <c r="F161" s="4" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="162" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -4080,16 +4050,16 @@
       </c>
       <c r="B162" s="4"/>
       <c r="C162" s="8" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="D162" s="5">
-        <v>400</v>
+        <v>300</v>
       </c>
       <c r="E162" s="6" t="s">
         <v>7</v>
       </c>
       <c r="F162" s="4" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="163" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -4098,16 +4068,16 @@
       </c>
       <c r="B163" s="4"/>
       <c r="C163" s="8" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="D163" s="5">
-        <v>300</v>
+        <v>400</v>
       </c>
       <c r="E163" s="6" t="s">
         <v>7</v>
       </c>
       <c r="F163" s="4" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="164" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -4116,16 +4086,16 @@
       </c>
       <c r="B164" s="4"/>
       <c r="C164" s="8" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="D164" s="5">
-        <v>300</v>
+        <v>800</v>
       </c>
       <c r="E164" s="6" t="s">
         <v>7</v>
       </c>
       <c r="F164" s="4" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="165" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -4134,13 +4104,13 @@
       </c>
       <c r="B165" s="4"/>
       <c r="C165" s="8" t="s">
-        <v>210</v>
+        <v>61</v>
       </c>
       <c r="D165" s="5">
-        <v>800</v>
+        <v>4</v>
       </c>
       <c r="E165" s="6" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="F165" s="4" t="s">
         <v>62</v>
@@ -4152,16 +4122,16 @@
       </c>
       <c r="B166" s="4"/>
       <c r="C166" s="8" t="s">
-        <v>63</v>
-      </c>
-      <c r="D166" s="5">
-        <v>4</v>
+        <v>207</v>
+      </c>
+      <c r="D166" s="7">
+        <v>2713.44</v>
       </c>
       <c r="E166" s="6" t="s">
         <v>11</v>
       </c>
       <c r="F166" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="167" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -4170,16 +4140,16 @@
       </c>
       <c r="B167" s="4"/>
       <c r="C167" s="8" t="s">
-        <v>211</v>
-      </c>
-      <c r="D167" s="7">
-        <v>2713.44</v>
+        <v>208</v>
+      </c>
+      <c r="D167" s="5">
+        <v>35.28</v>
       </c>
       <c r="E167" s="6" t="s">
         <v>11</v>
       </c>
       <c r="F167" s="4" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="168" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -4188,16 +4158,16 @@
       </c>
       <c r="B168" s="4"/>
       <c r="C168" s="8" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="D168" s="5">
-        <v>35.28</v>
+        <v>66</v>
       </c>
       <c r="E168" s="6" t="s">
         <v>11</v>
       </c>
       <c r="F168" s="4" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="169" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -4206,16 +4176,16 @@
       </c>
       <c r="B169" s="4"/>
       <c r="C169" s="8" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="D169" s="5">
-        <v>66</v>
+        <v>5.82</v>
       </c>
       <c r="E169" s="6" t="s">
         <v>11</v>
       </c>
       <c r="F169" s="4" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="170" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -4224,16 +4194,16 @@
       </c>
       <c r="B170" s="4"/>
       <c r="C170" s="8" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="D170" s="5">
-        <v>5.82</v>
+        <v>103.74</v>
       </c>
       <c r="E170" s="6" t="s">
         <v>11</v>
       </c>
       <c r="F170" s="4" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="171" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -4242,52 +4212,52 @@
       </c>
       <c r="B171" s="4"/>
       <c r="C171" s="8" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="D171" s="5">
-        <v>103.74</v>
+        <v>20.22</v>
       </c>
       <c r="E171" s="6" t="s">
         <v>11</v>
       </c>
       <c r="F171" s="4" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="172" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="172" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A172" s="3">
         <v>171</v>
       </c>
       <c r="B172" s="4"/>
       <c r="C172" s="8" t="s">
-        <v>216</v>
+        <v>64</v>
       </c>
       <c r="D172" s="5">
-        <v>20.22</v>
+        <v>612</v>
       </c>
       <c r="E172" s="6" t="s">
-        <v>11</v>
+        <v>65</v>
       </c>
       <c r="F172" s="4" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="173" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="173" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A173" s="3">
         <v>172</v>
       </c>
       <c r="B173" s="4"/>
       <c r="C173" s="8" t="s">
-        <v>66</v>
+        <v>213</v>
       </c>
       <c r="D173" s="5">
-        <v>612</v>
+        <v>19.5</v>
       </c>
       <c r="E173" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F173" s="4" t="s">
         <v>67</v>
-      </c>
-      <c r="F173" s="4" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="174" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -4296,16 +4266,16 @@
       </c>
       <c r="B174" s="4"/>
       <c r="C174" s="8" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="D174" s="5">
-        <v>19.5</v>
+        <v>1.8</v>
       </c>
       <c r="E174" s="6" t="s">
         <v>11</v>
       </c>
       <c r="F174" s="4" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="175" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -4314,16 +4284,16 @@
       </c>
       <c r="B175" s="4"/>
       <c r="C175" s="8" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="D175" s="5">
-        <v>1.8</v>
+        <v>4</v>
       </c>
       <c r="E175" s="6" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="F175" s="4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="176" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -4332,16 +4302,16 @@
       </c>
       <c r="B176" s="4"/>
       <c r="C176" s="8" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="D176" s="5">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E176" s="6" t="s">
         <v>7</v>
       </c>
       <c r="F176" s="4" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="177" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -4350,16 +4320,16 @@
       </c>
       <c r="B177" s="4"/>
       <c r="C177" s="8" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
       <c r="D177" s="5">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E177" s="6" t="s">
         <v>7</v>
       </c>
       <c r="F177" s="4" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="178" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -4368,7 +4338,7 @@
       </c>
       <c r="B178" s="4"/>
       <c r="C178" s="8" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="D178" s="5">
         <v>6</v>
@@ -4377,7 +4347,7 @@
         <v>7</v>
       </c>
       <c r="F178" s="4" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="179" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -4386,16 +4356,16 @@
       </c>
       <c r="B179" s="4"/>
       <c r="C179" s="8" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
       <c r="D179" s="5">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E179" s="6" t="s">
         <v>7</v>
       </c>
       <c r="F179" s="4" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="180" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -4404,34 +4374,34 @@
       </c>
       <c r="B180" s="4"/>
       <c r="C180" s="8" t="s">
-        <v>233</v>
+        <v>219</v>
       </c>
       <c r="D180" s="5">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E180" s="6" t="s">
         <v>7</v>
       </c>
       <c r="F180" s="4" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="181" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="181" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A181" s="3">
         <v>180</v>
       </c>
       <c r="B181" s="4"/>
       <c r="C181" s="8" t="s">
-        <v>223</v>
+        <v>197</v>
       </c>
       <c r="D181" s="5">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E181" s="6" t="s">
         <v>7</v>
       </c>
       <c r="F181" s="4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="182" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -4440,16 +4410,16 @@
       </c>
       <c r="B182" s="4"/>
       <c r="C182" s="8" t="s">
-        <v>71</v>
+        <v>220</v>
       </c>
       <c r="D182" s="5">
         <v>1</v>
       </c>
       <c r="E182" s="6" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="F182" s="4" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="183" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -4458,106 +4428,106 @@
       </c>
       <c r="B183" s="4"/>
       <c r="C183" s="8" t="s">
-        <v>73</v>
+        <v>221</v>
       </c>
       <c r="D183" s="5">
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="E183" s="6" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="F183" s="4" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="184" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="184" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A184" s="3">
         <v>183</v>
       </c>
       <c r="B184" s="4"/>
       <c r="C184" s="8" t="s">
-        <v>205</v>
-      </c>
-      <c r="D184" s="5">
-        <v>2</v>
+        <v>222</v>
+      </c>
+      <c r="D184" s="7">
+        <v>200000</v>
       </c>
       <c r="E184" s="6" t="s">
-        <v>7</v>
+        <v>24</v>
       </c>
       <c r="F184" s="4" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="185" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="185" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A185" s="3">
         <v>184</v>
       </c>
       <c r="B185" s="4"/>
       <c r="C185" s="8" t="s">
-        <v>224</v>
+        <v>72</v>
       </c>
       <c r="D185" s="5">
-        <v>100</v>
+        <v>3</v>
       </c>
       <c r="E185" s="6" t="s">
         <v>7</v>
       </c>
       <c r="F185" s="4" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="186" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="186" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A186" s="3">
         <v>185</v>
       </c>
       <c r="B186" s="4"/>
       <c r="C186" s="8" t="s">
-        <v>225</v>
+        <v>74</v>
       </c>
       <c r="D186" s="5">
-        <v>100</v>
+        <v>3</v>
       </c>
       <c r="E186" s="6" t="s">
         <v>7</v>
       </c>
       <c r="F186" s="4" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="187" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="187" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A187" s="3">
         <v>186</v>
       </c>
       <c r="B187" s="4"/>
       <c r="C187" s="8" t="s">
-        <v>226</v>
+        <v>76</v>
       </c>
       <c r="D187" s="5">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="E187" s="6" t="s">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="F187" s="4" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="188" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="188" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A188" s="3">
         <v>187</v>
       </c>
       <c r="B188" s="4"/>
       <c r="C188" s="8" t="s">
-        <v>227</v>
+        <v>77</v>
       </c>
       <c r="D188" s="5">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E188" s="6" t="s">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="F188" s="4" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="189" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -4566,178 +4536,34 @@
       </c>
       <c r="B189" s="4"/>
       <c r="C189" s="8" t="s">
-        <v>228</v>
+        <v>78</v>
       </c>
       <c r="D189" s="5">
-        <v>100</v>
+        <v>2</v>
       </c>
       <c r="E189" s="6" t="s">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="F189" s="4" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="190" spans="1:6" ht="35.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="190" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A190" s="3">
         <v>189</v>
       </c>
       <c r="B190" s="4"/>
       <c r="C190" s="8" t="s">
-        <v>229</v>
+        <v>79</v>
       </c>
       <c r="D190" s="5">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E190" s="6" t="s">
-        <v>77</v>
+        <v>15</v>
       </c>
       <c r="F190" s="4" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="191" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A191" s="3">
-        <v>190</v>
-      </c>
-      <c r="B191" s="4"/>
-      <c r="C191" s="8" t="s">
-        <v>78</v>
-      </c>
-      <c r="D191" s="5">
-        <v>36</v>
-      </c>
-      <c r="E191" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="F191" s="4" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="192" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A192" s="3">
-        <v>191</v>
-      </c>
-      <c r="B192" s="4"/>
-      <c r="C192" s="8" t="s">
-        <v>80</v>
-      </c>
-      <c r="D192" s="5">
-        <v>18</v>
-      </c>
-      <c r="E192" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="F192" s="4" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="193" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A193" s="3">
-        <v>192</v>
-      </c>
-      <c r="B193" s="4"/>
-      <c r="C193" s="8" t="s">
-        <v>230</v>
-      </c>
-      <c r="D193" s="5">
-        <v>36</v>
-      </c>
-      <c r="E193" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="F193" s="4" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="194" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A194" s="3">
-        <v>193</v>
-      </c>
-      <c r="B194" s="4"/>
-      <c r="C194" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="D194" s="5">
-        <v>18</v>
-      </c>
-      <c r="E194" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="F194" s="4" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="195" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A195" s="3">
-        <v>194</v>
-      </c>
-      <c r="B195" s="4"/>
-      <c r="C195" s="8" t="s">
-        <v>82</v>
-      </c>
-      <c r="D195" s="5">
-        <v>36</v>
-      </c>
-      <c r="E195" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="F195" s="4" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="196" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A196" s="3">
-        <v>195</v>
-      </c>
-      <c r="B196" s="4"/>
-      <c r="C196" s="8" t="s">
-        <v>83</v>
-      </c>
-      <c r="D196" s="5">
-        <v>18</v>
-      </c>
-      <c r="E196" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="F196" s="4" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="197" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A197" s="3">
-        <v>196</v>
-      </c>
-      <c r="B197" s="4"/>
-      <c r="C197" s="8" t="s">
-        <v>231</v>
-      </c>
-      <c r="D197" s="5">
-        <v>36</v>
-      </c>
-      <c r="E197" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="F197" s="4" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="198" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A198" s="3">
-        <v>197</v>
-      </c>
-      <c r="B198" s="4"/>
-      <c r="C198" s="8" t="s">
-        <v>232</v>
-      </c>
-      <c r="D198" s="5">
-        <v>36</v>
-      </c>
-      <c r="E198" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="F198" s="4" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
     </row>
   </sheetData>

</xml_diff>